<commit_message>
Incluir o apontamento do ponto de agosto nas três lojas
Nova aba PONTO AGO.26 em cada arquivo, com as ocorrências do mês e o
cálculo a partir do salário-hora. Os totais alimentam por SUMIFS as
linhas HORAS EXTRAS e ADICIONAL NOTURNO do holerite.

Arraial: EDEY 24 horas extras; NATI 17 horas noturnas e o feriado de
15/08; CAMILA, SARA e VALÉRIA o feriado de 15/08; VALÉRIA (2) e AGNOR
(3) madrugadas com folga, à espera das horas; DEAN com folga
compensatória, sem valor a pagar.

Trancoso: INIURLE com 40 horas extras. A conta confirma que os R$ 442,09
lançados em julho correspondem a 40 horas no salário de R$ 1.621,00 —
a observação sobre possível cópia de célula foi removida.

Parâmetros novos: horas mensais, adicional de hora extra, adicional
noturno e dias para o salário-dia.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2n4hj3F39Ez9XRrPSJYG5
</commit_message>
<xml_diff>
--- a/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_CENTRO_pgto_05-09-2026.xlsx
+++ b/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_CENTRO_pgto_05-09-2026.xlsx
@@ -14,7 +14,8 @@
     <sheet name="JULHO.26 REVISADO" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="LISTA CONTABILIDADE" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="GANHOS DO COLABORADOR" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="FOLGUISTAS" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="PONTO AGO.26" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="FOLGUISTAS" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'BASE INOVAFARMA AGO.26'!$A$4:$J$10</definedName>
@@ -22,7 +23,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'JULHO.26 REVISADO'!$A$4:$I$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'LISTA CONTABILIDADE'!$A$4:$E$153</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="6">'GANHOS DO COLABORADOR'!$A$1:$D$44</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'FOLGUISTAS'!$A$4:$H$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'PONTO AGO.26'!$A$4:$I$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'FOLGUISTAS'!$A$4:$H$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -215,7 +217,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -280,8 +282,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="11" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -305,6 +307,7 @@
     <xf numFmtId="0" fontId="15" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="16" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -671,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B44"/>
+  <dimension ref="A1:B45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -883,7 +886,7 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Horas extras e adicional noturno de agosto (apontamento do ponto).</t>
+          <t>Horas extras, adicional noturno e feriados trabalhados de agosto — lançar na aba PONTO AGO.26.</t>
         </is>
       </c>
     </row>
@@ -1032,6 +1035,14 @@
     <row r="44" ht="17" customHeight="1">
       <c r="A44" s="4" t="inlineStr"/>
       <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>PONTO AGO.26 — horas extras, adicional noturno e feriado trabalhado; alimenta o holerite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="17" customHeight="1">
+      <c r="A45" s="4" t="inlineStr"/>
+      <c r="B45" s="5" t="inlineStr">
         <is>
           <t>FOLGUISTAS — diárias de SERGIO e ANA CELIA para o contas a pagar (fora do holerite).</t>
         </is>
@@ -1059,7 +1070,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1248,54 +1259,114 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Multiplicador da comissão</t>
-        </is>
-      </c>
-      <c r="B16" s="12" t="n">
-        <v>1</v>
+          <t>Horas mensais (base do salário-hora)</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="n">
+        <v>220</v>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>1 = paga o valor apurado no InovaFarma, sem multiplicador.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>INSS / IRRF</t>
+          <t>Salário-hora = salário base ÷ 220.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Adicional de hora extra</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>50% sobre a hora normal (hora extra = salário-hora × 1,5).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>INSS</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>a calcular</t>
-        </is>
+          <t>Adicional noturno</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="n">
+        <v>0.2</v>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Calculado pela contabilidade sobre o total de proventos (tabela progressiva vigente).</t>
+          <t>20% sobre a hora normal, nas horas entre 22h e 5h.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
+          <t>Dias do mês para o salário-dia</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Salário-dia = salário base ÷ 30. Usado no feriado trabalhado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Multiplicador da comissão</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>1 = paga o valor apurado no InovaFarma, sem multiplicador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>INSS / IRRF</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>INSS</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>a calcular</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Calculado pela contabilidade sobre o total de proventos (tabela progressiva vigente).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
           <t>IRRF</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>a calcular</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="C23" s="9" t="inlineStr">
         <is>
           <t>Calculado pela contabilidade após dedução do INSS e dependentes.</t>
         </is>
@@ -1306,7 +1377,7 @@
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A21:C21"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
@@ -1933,19 +2004,37 @@
           <t>ADICIONAL NOTURNO</t>
         </is>
       </c>
-      <c r="B7" s="34" t="n"/>
-      <c r="C7" s="34" t="n"/>
-      <c r="D7" s="34" t="n"/>
-      <c r="E7" s="34" t="n"/>
-      <c r="F7" s="34" t="n"/>
-      <c r="G7" s="34" t="n"/>
+      <c r="B7" s="34">
+        <f>SUMIFS('PONTO AGO.26'!$G$5:$G$12,'PONTO AGO.26'!$A$5:$A$12,B$4,'PONTO AGO.26'!$H$5:$H$12,"ADICIONAL NOTURNO")</f>
+        <v/>
+      </c>
+      <c r="C7" s="34">
+        <f>SUMIFS('PONTO AGO.26'!$G$5:$G$12,'PONTO AGO.26'!$A$5:$A$12,C$4,'PONTO AGO.26'!$H$5:$H$12,"ADICIONAL NOTURNO")</f>
+        <v/>
+      </c>
+      <c r="D7" s="34">
+        <f>SUMIFS('PONTO AGO.26'!$G$5:$G$12,'PONTO AGO.26'!$A$5:$A$12,D$4,'PONTO AGO.26'!$H$5:$H$12,"ADICIONAL NOTURNO")</f>
+        <v/>
+      </c>
+      <c r="E7" s="34">
+        <f>SUMIFS('PONTO AGO.26'!$G$5:$G$12,'PONTO AGO.26'!$A$5:$A$12,E$4,'PONTO AGO.26'!$H$5:$H$12,"ADICIONAL NOTURNO")</f>
+        <v/>
+      </c>
+      <c r="F7" s="34">
+        <f>SUMIFS('PONTO AGO.26'!$G$5:$G$12,'PONTO AGO.26'!$A$5:$A$12,F$4,'PONTO AGO.26'!$H$5:$H$12,"ADICIONAL NOTURNO")</f>
+        <v/>
+      </c>
+      <c r="G7" s="34">
+        <f>SUMIFS('PONTO AGO.26'!$G$5:$G$12,'PONTO AGO.26'!$A$5:$A$12,G$4,'PONTO AGO.26'!$H$5:$H$12,"ADICIONAL NOTURNO")</f>
+        <v/>
+      </c>
       <c r="H7" s="20">
         <f>SUM(B7:G7)</f>
         <v/>
       </c>
       <c r="I7" s="33" t="inlineStr">
         <is>
-          <t>Conforme apontamento do ponto.</t>
+          <t>Somado automaticamente da aba PONTO AGO.26 (apontamento de agosto/2026). Para mudar, edite lá.</t>
         </is>
       </c>
     </row>
@@ -1955,19 +2044,37 @@
           <t>HORAS EXTRAS</t>
         </is>
       </c>
-      <c r="B8" s="34" t="n"/>
-      <c r="C8" s="34" t="n"/>
-      <c r="D8" s="34" t="n"/>
-      <c r="E8" s="34" t="n"/>
-      <c r="F8" s="34" t="n"/>
-      <c r="G8" s="34" t="n"/>
+      <c r="B8" s="34">
+        <f>SUMIFS('PONTO AGO.26'!$G$5:$G$12,'PONTO AGO.26'!$A$5:$A$12,B$4,'PONTO AGO.26'!$H$5:$H$12,"HORAS EXTRAS")</f>
+        <v/>
+      </c>
+      <c r="C8" s="34">
+        <f>SUMIFS('PONTO AGO.26'!$G$5:$G$12,'PONTO AGO.26'!$A$5:$A$12,C$4,'PONTO AGO.26'!$H$5:$H$12,"HORAS EXTRAS")</f>
+        <v/>
+      </c>
+      <c r="D8" s="34">
+        <f>SUMIFS('PONTO AGO.26'!$G$5:$G$12,'PONTO AGO.26'!$A$5:$A$12,D$4,'PONTO AGO.26'!$H$5:$H$12,"HORAS EXTRAS")</f>
+        <v/>
+      </c>
+      <c r="E8" s="34">
+        <f>SUMIFS('PONTO AGO.26'!$G$5:$G$12,'PONTO AGO.26'!$A$5:$A$12,E$4,'PONTO AGO.26'!$H$5:$H$12,"HORAS EXTRAS")</f>
+        <v/>
+      </c>
+      <c r="F8" s="34">
+        <f>SUMIFS('PONTO AGO.26'!$G$5:$G$12,'PONTO AGO.26'!$A$5:$A$12,F$4,'PONTO AGO.26'!$H$5:$H$12,"HORAS EXTRAS")</f>
+        <v/>
+      </c>
+      <c r="G8" s="34">
+        <f>SUMIFS('PONTO AGO.26'!$G$5:$G$12,'PONTO AGO.26'!$A$5:$A$12,G$4,'PONTO AGO.26'!$H$5:$H$12,"HORAS EXTRAS")</f>
+        <v/>
+      </c>
       <c r="H8" s="20">
         <f>SUM(B8:G8)</f>
         <v/>
       </c>
       <c r="I8" s="33" t="inlineStr">
         <is>
-          <t>PREENCHER com o apurado no ponto de agosto/2026.</t>
+          <t>Somado automaticamente da aba PONTO AGO.26 (apontamento de agosto/2026). Para mudar, edite lá.</t>
         </is>
       </c>
     </row>
@@ -1977,26 +2084,26 @@
           <t>COMISSÃO PRODUTOS (INOVAFARMA)</t>
         </is>
       </c>
-      <c r="B9" s="35" t="n">
+      <c r="B9" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="35">
-        <f>ROUND('BASE INOVAFARMA AGO.26'!F6*PARÂMETROS!$B$16,2)</f>
-        <v/>
-      </c>
-      <c r="D9" s="35">
-        <f>ROUND('BASE INOVAFARMA AGO.26'!F7*PARÂMETROS!$B$16,2)</f>
-        <v/>
-      </c>
-      <c r="E9" s="35">
-        <f>ROUND('BASE INOVAFARMA AGO.26'!F8*PARÂMETROS!$B$16,2)</f>
-        <v/>
-      </c>
-      <c r="F9" s="35">
-        <f>ROUND('BASE INOVAFARMA AGO.26'!F9*PARÂMETROS!$B$16,2)</f>
-        <v/>
-      </c>
-      <c r="G9" s="35" t="n">
+      <c r="C9" s="34">
+        <f>ROUND('BASE INOVAFARMA AGO.26'!F6*PARÂMETROS!$B$20,2)</f>
+        <v/>
+      </c>
+      <c r="D9" s="34">
+        <f>ROUND('BASE INOVAFARMA AGO.26'!F7*PARÂMETROS!$B$20,2)</f>
+        <v/>
+      </c>
+      <c r="E9" s="34">
+        <f>ROUND('BASE INOVAFARMA AGO.26'!F8*PARÂMETROS!$B$20,2)</f>
+        <v/>
+      </c>
+      <c r="F9" s="34">
+        <f>ROUND('BASE INOVAFARMA AGO.26'!F9*PARÂMETROS!$B$20,2)</f>
+        <v/>
+      </c>
+      <c r="G9" s="34" t="n">
         <v>0</v>
       </c>
       <c r="H9" s="20">
@@ -2015,12 +2122,12 @@
           <t>COMPLEMENTO / COMISSÃO PDV</t>
         </is>
       </c>
-      <c r="B10" s="34" t="n"/>
-      <c r="C10" s="34" t="n"/>
-      <c r="D10" s="34" t="n"/>
-      <c r="E10" s="34" t="n"/>
-      <c r="F10" s="34" t="n"/>
-      <c r="G10" s="34" t="n"/>
+      <c r="B10" s="35" t="n"/>
+      <c r="C10" s="35" t="n"/>
+      <c r="D10" s="35" t="n"/>
+      <c r="E10" s="35" t="n"/>
+      <c r="F10" s="35" t="n"/>
+      <c r="G10" s="35" t="n"/>
       <c r="H10" s="20">
         <f>SUM(B10:G10)</f>
         <v/>
@@ -2115,12 +2222,12 @@
           <t>AUXÍLIO GERÊNCIA</t>
         </is>
       </c>
-      <c r="B13" s="34" t="n"/>
-      <c r="C13" s="34" t="n"/>
-      <c r="D13" s="34" t="n"/>
-      <c r="E13" s="34" t="n"/>
-      <c r="F13" s="34" t="n"/>
-      <c r="G13" s="34" t="n"/>
+      <c r="B13" s="35" t="n"/>
+      <c r="C13" s="35" t="n"/>
+      <c r="D13" s="35" t="n"/>
+      <c r="E13" s="35" t="n"/>
+      <c r="F13" s="35" t="n"/>
+      <c r="G13" s="35" t="n"/>
       <c r="H13" s="20">
         <f>SUM(B13:G13)</f>
         <v/>
@@ -2137,12 +2244,12 @@
           <t>ADICIONAL PRÊMIO META CAIXA</t>
         </is>
       </c>
-      <c r="B14" s="34" t="n"/>
-      <c r="C14" s="34" t="n"/>
-      <c r="D14" s="34" t="n"/>
-      <c r="E14" s="34" t="n"/>
-      <c r="F14" s="34" t="n"/>
-      <c r="G14" s="34" t="n"/>
+      <c r="B14" s="35" t="n"/>
+      <c r="C14" s="35" t="n"/>
+      <c r="D14" s="35" t="n"/>
+      <c r="E14" s="35" t="n"/>
+      <c r="F14" s="35" t="n"/>
+      <c r="G14" s="35" t="n"/>
       <c r="H14" s="20">
         <f>SUM(B14:G14)</f>
         <v/>
@@ -2159,12 +2266,12 @@
           <t>PRÊMIO COTA GERAL</t>
         </is>
       </c>
-      <c r="B15" s="34" t="n"/>
-      <c r="C15" s="34" t="n"/>
-      <c r="D15" s="34" t="n"/>
-      <c r="E15" s="34" t="n"/>
-      <c r="F15" s="34" t="n"/>
-      <c r="G15" s="34" t="n"/>
+      <c r="B15" s="35" t="n"/>
+      <c r="C15" s="35" t="n"/>
+      <c r="D15" s="35" t="n"/>
+      <c r="E15" s="35" t="n"/>
+      <c r="F15" s="35" t="n"/>
+      <c r="G15" s="35" t="n"/>
       <c r="H15" s="20">
         <f>SUM(B15:G15)</f>
         <v/>
@@ -2181,12 +2288,12 @@
           <t>PRÊMIO PRÉ-VENCIDOS</t>
         </is>
       </c>
-      <c r="B16" s="34" t="n"/>
-      <c r="C16" s="34" t="n"/>
-      <c r="D16" s="34" t="n"/>
-      <c r="E16" s="34" t="n"/>
-      <c r="F16" s="34" t="n"/>
-      <c r="G16" s="34" t="n"/>
+      <c r="B16" s="35" t="n"/>
+      <c r="C16" s="35" t="n"/>
+      <c r="D16" s="35" t="n"/>
+      <c r="E16" s="35" t="n"/>
+      <c r="F16" s="35" t="n"/>
+      <c r="G16" s="35" t="n"/>
       <c r="H16" s="20">
         <f>SUM(B16:G16)</f>
         <v/>
@@ -2203,12 +2310,12 @@
           <t>FÉRIAS (DIAS GOZADOS)</t>
         </is>
       </c>
-      <c r="B17" s="34" t="n"/>
-      <c r="C17" s="34" t="n"/>
-      <c r="D17" s="34" t="n"/>
-      <c r="E17" s="34" t="n"/>
-      <c r="F17" s="34" t="n"/>
-      <c r="G17" s="34" t="n"/>
+      <c r="B17" s="35" t="n"/>
+      <c r="C17" s="35" t="n"/>
+      <c r="D17" s="35" t="n"/>
+      <c r="E17" s="35" t="n"/>
+      <c r="F17" s="35" t="n"/>
+      <c r="G17" s="35" t="n"/>
       <c r="H17" s="20">
         <f>SUM(B17:G17)</f>
         <v/>
@@ -2225,12 +2332,12 @@
           <t>1/3 CONSTITUCIONAL DE FÉRIAS</t>
         </is>
       </c>
-      <c r="B18" s="34" t="n"/>
-      <c r="C18" s="34" t="n"/>
-      <c r="D18" s="34" t="n"/>
-      <c r="E18" s="34" t="n"/>
-      <c r="F18" s="34" t="n"/>
-      <c r="G18" s="34" t="n"/>
+      <c r="B18" s="35" t="n"/>
+      <c r="C18" s="35" t="n"/>
+      <c r="D18" s="35" t="n"/>
+      <c r="E18" s="35" t="n"/>
+      <c r="F18" s="35" t="n"/>
+      <c r="G18" s="35" t="n"/>
       <c r="H18" s="20">
         <f>SUM(B18:G18)</f>
         <v/>
@@ -2247,27 +2354,27 @@
           <t>INCENTIVO APLICAÇÕES</t>
         </is>
       </c>
-      <c r="B19" s="35">
+      <c r="B19" s="34">
         <f>'BASE INOVAFARMA AGO.26'!G5</f>
         <v/>
       </c>
-      <c r="C19" s="35">
+      <c r="C19" s="34">
         <f>'BASE INOVAFARMA AGO.26'!G6</f>
         <v/>
       </c>
-      <c r="D19" s="35">
+      <c r="D19" s="34">
         <f>'BASE INOVAFARMA AGO.26'!G7</f>
         <v/>
       </c>
-      <c r="E19" s="35">
+      <c r="E19" s="34">
         <f>'BASE INOVAFARMA AGO.26'!G8</f>
         <v/>
       </c>
-      <c r="F19" s="35">
+      <c r="F19" s="34">
         <f>'BASE INOVAFARMA AGO.26'!G9</f>
         <v/>
       </c>
-      <c r="G19" s="35">
+      <c r="G19" s="34">
         <f>'BASE INOVAFARMA AGO.26'!G10</f>
         <v/>
       </c>
@@ -2287,27 +2394,27 @@
           <t>INCENTIVO VITAMINAS</t>
         </is>
       </c>
-      <c r="B20" s="35">
+      <c r="B20" s="34">
         <f>'BASE INOVAFARMA AGO.26'!H5</f>
         <v/>
       </c>
-      <c r="C20" s="35">
+      <c r="C20" s="34">
         <f>'BASE INOVAFARMA AGO.26'!H6</f>
         <v/>
       </c>
-      <c r="D20" s="35">
+      <c r="D20" s="34">
         <f>'BASE INOVAFARMA AGO.26'!H7</f>
         <v/>
       </c>
-      <c r="E20" s="35">
+      <c r="E20" s="34">
         <f>'BASE INOVAFARMA AGO.26'!H8</f>
         <v/>
       </c>
-      <c r="F20" s="35">
+      <c r="F20" s="34">
         <f>'BASE INOVAFARMA AGO.26'!H9</f>
         <v/>
       </c>
-      <c r="G20" s="35">
+      <c r="G20" s="34">
         <f>'BASE INOVAFARMA AGO.26'!H10</f>
         <v/>
       </c>
@@ -2327,27 +2434,27 @@
           <t>OUTROS INCENTIVOS</t>
         </is>
       </c>
-      <c r="B21" s="35">
+      <c r="B21" s="34">
         <f>'BASE INOVAFARMA AGO.26'!I5</f>
         <v/>
       </c>
-      <c r="C21" s="35">
+      <c r="C21" s="34">
         <f>'BASE INOVAFARMA AGO.26'!I6</f>
         <v/>
       </c>
-      <c r="D21" s="35">
+      <c r="D21" s="34">
         <f>'BASE INOVAFARMA AGO.26'!I7</f>
         <v/>
       </c>
-      <c r="E21" s="35">
+      <c r="E21" s="34">
         <f>'BASE INOVAFARMA AGO.26'!I8</f>
         <v/>
       </c>
-      <c r="F21" s="35">
+      <c r="F21" s="34">
         <f>'BASE INOVAFARMA AGO.26'!I9</f>
         <v/>
       </c>
-      <c r="G21" s="35">
+      <c r="G21" s="34">
         <f>'BASE INOVAFARMA AGO.26'!I10</f>
         <v/>
       </c>
@@ -2422,12 +2529,12 @@
           <t>ADIANTAMENTO / VALES</t>
         </is>
       </c>
-      <c r="B24" s="34" t="n"/>
-      <c r="C24" s="34" t="n"/>
-      <c r="D24" s="34" t="n"/>
-      <c r="E24" s="34" t="n"/>
-      <c r="F24" s="34" t="n"/>
-      <c r="G24" s="34" t="n"/>
+      <c r="B24" s="35" t="n"/>
+      <c r="C24" s="35" t="n"/>
+      <c r="D24" s="35" t="n"/>
+      <c r="E24" s="35" t="n"/>
+      <c r="F24" s="35" t="n"/>
+      <c r="G24" s="35" t="n"/>
       <c r="H24" s="20">
         <f>SUM(B24:G24)</f>
         <v/>
@@ -2484,12 +2591,12 @@
           <t>CONVÊNIO</t>
         </is>
       </c>
-      <c r="B26" s="34" t="n"/>
-      <c r="C26" s="34" t="n"/>
-      <c r="D26" s="34" t="n"/>
-      <c r="E26" s="34" t="n"/>
-      <c r="F26" s="34" t="n"/>
-      <c r="G26" s="34" t="n"/>
+      <c r="B26" s="35" t="n"/>
+      <c r="C26" s="35" t="n"/>
+      <c r="D26" s="35" t="n"/>
+      <c r="E26" s="35" t="n"/>
+      <c r="F26" s="35" t="n"/>
+      <c r="G26" s="35" t="n"/>
       <c r="H26" s="20">
         <f>SUM(B26:G26)</f>
         <v/>
@@ -2506,12 +2613,12 @@
           <t>DESCONTO FALTAS / ATRASOS</t>
         </is>
       </c>
-      <c r="B27" s="34" t="n"/>
-      <c r="C27" s="34" t="n"/>
-      <c r="D27" s="34" t="n"/>
-      <c r="E27" s="34" t="n"/>
-      <c r="F27" s="34" t="n"/>
-      <c r="G27" s="34" t="n"/>
+      <c r="B27" s="35" t="n"/>
+      <c r="C27" s="35" t="n"/>
+      <c r="D27" s="35" t="n"/>
+      <c r="E27" s="35" t="n"/>
+      <c r="F27" s="35" t="n"/>
+      <c r="G27" s="35" t="n"/>
       <c r="H27" s="20">
         <f>SUM(B27:G27)</f>
         <v/>
@@ -2558,12 +2665,12 @@
           <t>DESCONTO INSS</t>
         </is>
       </c>
-      <c r="B29" s="34" t="n"/>
-      <c r="C29" s="34" t="n"/>
-      <c r="D29" s="34" t="n"/>
-      <c r="E29" s="34" t="n"/>
-      <c r="F29" s="34" t="n"/>
-      <c r="G29" s="34" t="n"/>
+      <c r="B29" s="35" t="n"/>
+      <c r="C29" s="35" t="n"/>
+      <c r="D29" s="35" t="n"/>
+      <c r="E29" s="35" t="n"/>
+      <c r="F29" s="35" t="n"/>
+      <c r="G29" s="35" t="n"/>
       <c r="H29" s="20">
         <f>SUM(B29:G29)</f>
         <v/>
@@ -2580,12 +2687,12 @@
           <t>DESCONTO IRRF</t>
         </is>
       </c>
-      <c r="B30" s="34" t="n"/>
-      <c r="C30" s="34" t="n"/>
-      <c r="D30" s="34" t="n"/>
-      <c r="E30" s="34" t="n"/>
-      <c r="F30" s="34" t="n"/>
-      <c r="G30" s="34" t="n"/>
+      <c r="B30" s="35" t="n"/>
+      <c r="C30" s="35" t="n"/>
+      <c r="D30" s="35" t="n"/>
+      <c r="E30" s="35" t="n"/>
+      <c r="F30" s="35" t="n"/>
+      <c r="G30" s="35" t="n"/>
       <c r="H30" s="20">
         <f>SUM(B30:G30)</f>
         <v/>
@@ -2708,12 +2815,12 @@
           <t>VALE TRANSPORTE (compra set/26)</t>
         </is>
       </c>
-      <c r="B35" s="34" t="n"/>
-      <c r="C35" s="34" t="n"/>
-      <c r="D35" s="34" t="n"/>
-      <c r="E35" s="34" t="n"/>
-      <c r="F35" s="34" t="n"/>
-      <c r="G35" s="34" t="n"/>
+      <c r="B35" s="35" t="n"/>
+      <c r="C35" s="35" t="n"/>
+      <c r="D35" s="35" t="n"/>
+      <c r="E35" s="35" t="n"/>
+      <c r="F35" s="35" t="n"/>
+      <c r="G35" s="35" t="n"/>
       <c r="H35" s="20">
         <f>SUM(B35:G35)</f>
         <v/>
@@ -2730,12 +2837,12 @@
           <t>VALE ALIMENTAÇÃO FERIADOS E DOMINGOS</t>
         </is>
       </c>
-      <c r="B36" s="34" t="n"/>
-      <c r="C36" s="34" t="n"/>
-      <c r="D36" s="34" t="n"/>
-      <c r="E36" s="34" t="n"/>
-      <c r="F36" s="34" t="n"/>
-      <c r="G36" s="34" t="n"/>
+      <c r="B36" s="35" t="n"/>
+      <c r="C36" s="35" t="n"/>
+      <c r="D36" s="35" t="n"/>
+      <c r="E36" s="35" t="n"/>
+      <c r="F36" s="35" t="n"/>
+      <c r="G36" s="35" t="n"/>
       <c r="H36" s="20">
         <f>SUM(B36:G36)</f>
         <v/>
@@ -2919,22 +3026,22 @@
           <t>SALÁRIO BASE</t>
         </is>
       </c>
-      <c r="B6" s="34" t="n">
+      <c r="B6" s="35" t="n">
         <v>5648.41</v>
       </c>
-      <c r="C6" s="34" t="n">
+      <c r="C6" s="35" t="n">
         <v>1621</v>
       </c>
-      <c r="D6" s="34" t="n">
+      <c r="D6" s="35" t="n">
         <v>1621</v>
       </c>
-      <c r="E6" s="34" t="n">
+      <c r="E6" s="35" t="n">
         <v>1621</v>
       </c>
-      <c r="F6" s="34" t="n">
+      <c r="F6" s="35" t="n">
         <v>1621</v>
       </c>
-      <c r="G6" s="34" t="n">
+      <c r="G6" s="35" t="n">
         <v>1621</v>
       </c>
       <c r="H6" s="20">
@@ -2949,12 +3056,12 @@
           <t>ADICIONAL NOTURNO</t>
         </is>
       </c>
-      <c r="B7" s="34" t="n"/>
-      <c r="C7" s="34" t="n"/>
-      <c r="D7" s="34" t="n"/>
-      <c r="E7" s="34" t="n"/>
-      <c r="F7" s="34" t="n"/>
-      <c r="G7" s="34" t="n"/>
+      <c r="B7" s="35" t="n"/>
+      <c r="C7" s="35" t="n"/>
+      <c r="D7" s="35" t="n"/>
+      <c r="E7" s="35" t="n"/>
+      <c r="F7" s="35" t="n"/>
+      <c r="G7" s="35" t="n"/>
       <c r="H7" s="20">
         <f>SUM(B7:G7)</f>
         <v/>
@@ -2967,12 +3074,12 @@
           <t>HORAS EXTRAS</t>
         </is>
       </c>
-      <c r="B8" s="34" t="n"/>
-      <c r="C8" s="34" t="n"/>
-      <c r="D8" s="34" t="n"/>
-      <c r="E8" s="34" t="n"/>
-      <c r="F8" s="34" t="n"/>
-      <c r="G8" s="34" t="n"/>
+      <c r="B8" s="35" t="n"/>
+      <c r="C8" s="35" t="n"/>
+      <c r="D8" s="35" t="n"/>
+      <c r="E8" s="35" t="n"/>
+      <c r="F8" s="35" t="n"/>
+      <c r="G8" s="35" t="n"/>
       <c r="H8" s="20">
         <f>SUM(B8:G8)</f>
         <v/>
@@ -2985,20 +3092,20 @@
           <t>COMISSÃO PRODUTOS + PDV</t>
         </is>
       </c>
-      <c r="B9" s="34" t="n"/>
-      <c r="C9" s="34" t="n">
+      <c r="B9" s="35" t="n"/>
+      <c r="C9" s="35" t="n">
         <v>1400</v>
       </c>
-      <c r="D9" s="34" t="n">
+      <c r="D9" s="35" t="n">
         <v>100</v>
       </c>
-      <c r="E9" s="34" t="n">
+      <c r="E9" s="35" t="n">
         <v>1200</v>
       </c>
-      <c r="F9" s="34" t="n">
+      <c r="F9" s="35" t="n">
         <v>60</v>
       </c>
-      <c r="G9" s="34" t="n"/>
+      <c r="G9" s="35" t="n"/>
       <c r="H9" s="20">
         <f>SUM(B9:G9)</f>
         <v/>
@@ -3015,20 +3122,20 @@
           <t>REPOUSO REMUNERADO / DSR</t>
         </is>
       </c>
-      <c r="B10" s="34" t="n"/>
-      <c r="C10" s="34" t="n">
+      <c r="B10" s="35" t="n"/>
+      <c r="C10" s="35" t="n">
         <v>269.23</v>
       </c>
-      <c r="D10" s="34" t="n">
+      <c r="D10" s="35" t="n">
         <v>19.23</v>
       </c>
-      <c r="E10" s="34" t="n">
+      <c r="E10" s="35" t="n">
         <v>230.77</v>
       </c>
-      <c r="F10" s="34" t="n">
+      <c r="F10" s="35" t="n">
         <v>11.54</v>
       </c>
-      <c r="G10" s="34" t="n"/>
+      <c r="G10" s="35" t="n"/>
       <c r="H10" s="20">
         <f>SUM(B10:G10)</f>
         <v/>
@@ -3045,12 +3152,12 @@
           <t>AUXÍLIO GERÊNCIA</t>
         </is>
       </c>
-      <c r="B11" s="34" t="n"/>
-      <c r="C11" s="34" t="n"/>
-      <c r="D11" s="34" t="n"/>
-      <c r="E11" s="34" t="n"/>
-      <c r="F11" s="34" t="n"/>
-      <c r="G11" s="34" t="n"/>
+      <c r="B11" s="35" t="n"/>
+      <c r="C11" s="35" t="n"/>
+      <c r="D11" s="35" t="n"/>
+      <c r="E11" s="35" t="n"/>
+      <c r="F11" s="35" t="n"/>
+      <c r="G11" s="35" t="n"/>
       <c r="H11" s="20">
         <f>SUM(B11:G11)</f>
         <v/>
@@ -3063,20 +3170,20 @@
           <t>PRÊMIO COTA GERAL</t>
         </is>
       </c>
-      <c r="B12" s="34" t="n"/>
-      <c r="C12" s="34" t="n">
+      <c r="B12" s="35" t="n"/>
+      <c r="C12" s="35" t="n">
         <v>300</v>
       </c>
-      <c r="D12" s="34" t="n">
+      <c r="D12" s="35" t="n">
         <v>100</v>
       </c>
-      <c r="E12" s="34" t="n">
+      <c r="E12" s="35" t="n">
         <v>150</v>
       </c>
-      <c r="F12" s="34" t="n">
+      <c r="F12" s="35" t="n">
         <v>100</v>
       </c>
-      <c r="G12" s="34" t="n"/>
+      <c r="G12" s="35" t="n"/>
       <c r="H12" s="20">
         <f>SUM(B12:G12)</f>
         <v/>
@@ -3089,16 +3196,16 @@
           <t>PRÊMIO PRÉ-VENCIDOS</t>
         </is>
       </c>
-      <c r="B13" s="34" t="n"/>
-      <c r="C13" s="34" t="n">
+      <c r="B13" s="35" t="n"/>
+      <c r="C13" s="35" t="n">
         <v>250</v>
       </c>
-      <c r="D13" s="34" t="n"/>
-      <c r="E13" s="34" t="n">
+      <c r="D13" s="35" t="n"/>
+      <c r="E13" s="35" t="n">
         <v>100</v>
       </c>
-      <c r="F13" s="34" t="n"/>
-      <c r="G13" s="34" t="n"/>
+      <c r="F13" s="35" t="n"/>
+      <c r="G13" s="35" t="n"/>
       <c r="H13" s="20">
         <f>SUM(B13:G13)</f>
         <v/>
@@ -3111,12 +3218,12 @@
           <t>INCENTIVO APLICAÇÕES</t>
         </is>
       </c>
-      <c r="B14" s="34" t="n"/>
-      <c r="C14" s="34" t="n"/>
-      <c r="D14" s="34" t="n"/>
-      <c r="E14" s="34" t="n"/>
-      <c r="F14" s="34" t="n"/>
-      <c r="G14" s="34" t="n"/>
+      <c r="B14" s="35" t="n"/>
+      <c r="C14" s="35" t="n"/>
+      <c r="D14" s="35" t="n"/>
+      <c r="E14" s="35" t="n"/>
+      <c r="F14" s="35" t="n"/>
+      <c r="G14" s="35" t="n"/>
       <c r="H14" s="20">
         <f>SUM(B14:G14)</f>
         <v/>
@@ -3129,12 +3236,12 @@
           <t>INCENTIVO VITAMINAS</t>
         </is>
       </c>
-      <c r="B15" s="34" t="n"/>
-      <c r="C15" s="34" t="n"/>
-      <c r="D15" s="34" t="n"/>
-      <c r="E15" s="34" t="n"/>
-      <c r="F15" s="34" t="n"/>
-      <c r="G15" s="34" t="n"/>
+      <c r="B15" s="35" t="n"/>
+      <c r="C15" s="35" t="n"/>
+      <c r="D15" s="35" t="n"/>
+      <c r="E15" s="35" t="n"/>
+      <c r="F15" s="35" t="n"/>
+      <c r="G15" s="35" t="n"/>
       <c r="H15" s="20">
         <f>SUM(B15:G15)</f>
         <v/>
@@ -3198,18 +3305,18 @@
           <t>ADIANTAMENTO / VALES</t>
         </is>
       </c>
-      <c r="B18" s="34" t="n"/>
-      <c r="C18" s="34" t="n">
+      <c r="B18" s="35" t="n"/>
+      <c r="C18" s="35" t="n">
         <v>-1300</v>
       </c>
-      <c r="D18" s="34" t="n">
+      <c r="D18" s="35" t="n">
         <v>-700</v>
       </c>
-      <c r="E18" s="34" t="n">
+      <c r="E18" s="35" t="n">
         <v>-1000</v>
       </c>
-      <c r="F18" s="34" t="n"/>
-      <c r="G18" s="34" t="n"/>
+      <c r="F18" s="35" t="n"/>
+      <c r="G18" s="35" t="n"/>
       <c r="H18" s="20">
         <f>SUM(B18:G18)</f>
         <v/>
@@ -3222,18 +3329,18 @@
           <t>CONVÊNIO</t>
         </is>
       </c>
-      <c r="B19" s="34" t="n"/>
-      <c r="C19" s="34" t="n"/>
-      <c r="D19" s="34" t="n">
+      <c r="B19" s="35" t="n"/>
+      <c r="C19" s="35" t="n"/>
+      <c r="D19" s="35" t="n">
         <v>-400</v>
       </c>
-      <c r="E19" s="34" t="n">
+      <c r="E19" s="35" t="n">
         <v>-400</v>
       </c>
-      <c r="F19" s="34" t="n">
+      <c r="F19" s="35" t="n">
         <v>-200</v>
       </c>
-      <c r="G19" s="34" t="n"/>
+      <c r="G19" s="35" t="n"/>
       <c r="H19" s="20">
         <f>SUM(B19:G19)</f>
         <v/>
@@ -3246,12 +3353,12 @@
           <t>DESCONTO FALTAS</t>
         </is>
       </c>
-      <c r="B20" s="34" t="n"/>
-      <c r="C20" s="34" t="n"/>
-      <c r="D20" s="34" t="n"/>
-      <c r="E20" s="34" t="n"/>
-      <c r="F20" s="34" t="n"/>
-      <c r="G20" s="34" t="n"/>
+      <c r="B20" s="35" t="n"/>
+      <c r="C20" s="35" t="n"/>
+      <c r="D20" s="35" t="n"/>
+      <c r="E20" s="35" t="n"/>
+      <c r="F20" s="35" t="n"/>
+      <c r="G20" s="35" t="n"/>
       <c r="H20" s="20">
         <f>SUM(B20:G20)</f>
         <v/>
@@ -3264,20 +3371,20 @@
           <t>DESCONTO VALE TRANSPORTE 6%</t>
         </is>
       </c>
-      <c r="B21" s="34" t="n"/>
-      <c r="C21" s="34" t="n">
+      <c r="B21" s="35" t="n"/>
+      <c r="C21" s="35" t="n">
         <v>-84.29000000000001</v>
       </c>
-      <c r="D21" s="34" t="n">
+      <c r="D21" s="35" t="n">
         <v>-84.29000000000001</v>
       </c>
-      <c r="E21" s="34" t="n">
+      <c r="E21" s="35" t="n">
         <v>-74.29000000000001</v>
       </c>
-      <c r="F21" s="34" t="n">
+      <c r="F21" s="35" t="n">
         <v>-84.29000000000001</v>
       </c>
-      <c r="G21" s="34" t="n"/>
+      <c r="G21" s="35" t="n"/>
       <c r="H21" s="20">
         <f>SUM(B21:G21)</f>
         <v/>
@@ -3290,22 +3397,22 @@
           <t>DESCONTO INSS</t>
         </is>
       </c>
-      <c r="B22" s="34" t="n">
+      <c r="B22" s="35" t="n">
         <v>-592.27</v>
       </c>
-      <c r="C22" s="34" t="n">
+      <c r="C22" s="35" t="n">
         <v>-349.41</v>
       </c>
-      <c r="D22" s="34" t="n">
+      <c r="D22" s="35" t="n">
         <v>-141.3</v>
       </c>
-      <c r="E22" s="34" t="n">
+      <c r="E22" s="35" t="n">
         <v>-284.8</v>
       </c>
-      <c r="F22" s="34" t="n">
+      <c r="F22" s="35" t="n">
         <v>-137</v>
       </c>
-      <c r="G22" s="34" t="n"/>
+      <c r="G22" s="35" t="n"/>
       <c r="H22" s="20">
         <f>SUM(B22:G22)</f>
         <v/>
@@ -3318,14 +3425,14 @@
           <t>DESCONTO IRRF</t>
         </is>
       </c>
-      <c r="B23" s="34" t="n">
+      <c r="B23" s="35" t="n">
         <v>-251.04</v>
       </c>
-      <c r="C23" s="34" t="n"/>
-      <c r="D23" s="34" t="n"/>
-      <c r="E23" s="34" t="n"/>
-      <c r="F23" s="34" t="n"/>
-      <c r="G23" s="34" t="n"/>
+      <c r="C23" s="35" t="n"/>
+      <c r="D23" s="35" t="n"/>
+      <c r="E23" s="35" t="n"/>
+      <c r="F23" s="35" t="n"/>
+      <c r="G23" s="35" t="n"/>
       <c r="H23" s="20">
         <f>SUM(B23:G23)</f>
         <v/>
@@ -3425,22 +3532,22 @@
           <t>SALDO FINAL DA PLANILHA ORIGINAL</t>
         </is>
       </c>
-      <c r="B27" s="34" t="n">
+      <c r="B27" s="35" t="n">
         <v>4805.1</v>
       </c>
-      <c r="C27" s="34" t="n">
+      <c r="C27" s="35" t="n">
         <v>2106.53</v>
       </c>
-      <c r="D27" s="34" t="n">
+      <c r="D27" s="35" t="n">
         <v>514.64</v>
       </c>
-      <c r="E27" s="34" t="n">
+      <c r="E27" s="35" t="n">
         <v>1542.68</v>
       </c>
-      <c r="F27" s="34" t="n">
+      <c r="F27" s="35" t="n">
         <v>1371.25</v>
       </c>
-      <c r="G27" s="34" t="n">
+      <c r="G27" s="35" t="n">
         <v>1621</v>
       </c>
       <c r="H27" s="20">
@@ -3649,18 +3756,18 @@
           <t>VALE TRANSPORTE</t>
         </is>
       </c>
-      <c r="B34" s="34" t="n"/>
-      <c r="C34" s="34" t="n">
+      <c r="B34" s="35" t="n"/>
+      <c r="C34" s="35" t="n">
         <v>270</v>
       </c>
-      <c r="D34" s="34" t="n"/>
-      <c r="E34" s="34" t="n">
+      <c r="D34" s="35" t="n"/>
+      <c r="E34" s="35" t="n">
         <v>260</v>
       </c>
-      <c r="F34" s="34" t="n">
+      <c r="F34" s="35" t="n">
         <v>260</v>
       </c>
-      <c r="G34" s="34" t="n">
+      <c r="G34" s="35" t="n">
         <v>350</v>
       </c>
       <c r="H34" s="20">
@@ -3796,7 +3903,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D5" s="35">
+      <c r="D5" s="34">
         <f>'HOLERITE AGO.26'!B6</f>
         <v/>
       </c>
@@ -3818,7 +3925,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D6" s="35">
+      <c r="D6" s="34">
         <f>'HOLERITE AGO.26'!B7</f>
         <v/>
       </c>
@@ -3840,7 +3947,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D7" s="35">
+      <c r="D7" s="34">
         <f>'HOLERITE AGO.26'!B8</f>
         <v/>
       </c>
@@ -3862,7 +3969,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D8" s="35">
+      <c r="D8" s="34">
         <f>'HOLERITE AGO.26'!B11</f>
         <v/>
       </c>
@@ -3884,7 +3991,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D9" s="35">
+      <c r="D9" s="34">
         <f>'HOLERITE AGO.26'!B12</f>
         <v/>
       </c>
@@ -3906,7 +4013,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D10" s="35">
+      <c r="D10" s="34">
         <f>'HOLERITE AGO.26'!B13</f>
         <v/>
       </c>
@@ -3928,7 +4035,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D11" s="35">
+      <c r="D11" s="34">
         <f>'HOLERITE AGO.26'!B14</f>
         <v/>
       </c>
@@ -3950,7 +4057,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D12" s="35">
+      <c r="D12" s="34">
         <f>'HOLERITE AGO.26'!B15</f>
         <v/>
       </c>
@@ -3972,7 +4079,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D13" s="35">
+      <c r="D13" s="34">
         <f>'HOLERITE AGO.26'!B16</f>
         <v/>
       </c>
@@ -3994,7 +4101,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D14" s="35">
+      <c r="D14" s="34">
         <f>'HOLERITE AGO.26'!B17</f>
         <v/>
       </c>
@@ -4016,7 +4123,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D15" s="35">
+      <c r="D15" s="34">
         <f>'HOLERITE AGO.26'!B18</f>
         <v/>
       </c>
@@ -4038,7 +4145,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D16" s="35">
+      <c r="D16" s="34">
         <f>'HOLERITE AGO.26'!B19</f>
         <v/>
       </c>
@@ -4060,7 +4167,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D17" s="35">
+      <c r="D17" s="34">
         <f>'HOLERITE AGO.26'!B20</f>
         <v/>
       </c>
@@ -4082,7 +4189,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D18" s="35">
+      <c r="D18" s="34">
         <f>'HOLERITE AGO.26'!B21</f>
         <v/>
       </c>
@@ -4126,7 +4233,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D20" s="35">
+      <c r="D20" s="34">
         <f>'HOLERITE AGO.26'!B24</f>
         <v/>
       </c>
@@ -4148,7 +4255,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D21" s="35">
+      <c r="D21" s="34">
         <f>'HOLERITE AGO.26'!B25</f>
         <v/>
       </c>
@@ -4170,7 +4277,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D22" s="35">
+      <c r="D22" s="34">
         <f>'HOLERITE AGO.26'!B26</f>
         <v/>
       </c>
@@ -4192,7 +4299,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D23" s="35">
+      <c r="D23" s="34">
         <f>'HOLERITE AGO.26'!B27</f>
         <v/>
       </c>
@@ -4214,7 +4321,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D24" s="35">
+      <c r="D24" s="34">
         <f>'HOLERITE AGO.26'!B28</f>
         <v/>
       </c>
@@ -4236,7 +4343,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D25" s="35">
+      <c r="D25" s="34">
         <f>'HOLERITE AGO.26'!B29</f>
         <v/>
       </c>
@@ -4258,7 +4365,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D26" s="35">
+      <c r="D26" s="34">
         <f>'HOLERITE AGO.26'!B30</f>
         <v/>
       </c>
@@ -4324,7 +4431,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D30" s="35">
+      <c r="D30" s="34">
         <f>'HOLERITE AGO.26'!C6</f>
         <v/>
       </c>
@@ -4346,7 +4453,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D31" s="35">
+      <c r="D31" s="34">
         <f>'HOLERITE AGO.26'!C7</f>
         <v/>
       </c>
@@ -4368,7 +4475,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D32" s="35">
+      <c r="D32" s="34">
         <f>'HOLERITE AGO.26'!C8</f>
         <v/>
       </c>
@@ -4390,7 +4497,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D33" s="35">
+      <c r="D33" s="34">
         <f>'HOLERITE AGO.26'!C11</f>
         <v/>
       </c>
@@ -4412,7 +4519,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D34" s="35">
+      <c r="D34" s="34">
         <f>'HOLERITE AGO.26'!C12</f>
         <v/>
       </c>
@@ -4434,7 +4541,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D35" s="35">
+      <c r="D35" s="34">
         <f>'HOLERITE AGO.26'!C13</f>
         <v/>
       </c>
@@ -4456,7 +4563,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D36" s="35">
+      <c r="D36" s="34">
         <f>'HOLERITE AGO.26'!C14</f>
         <v/>
       </c>
@@ -4478,7 +4585,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D37" s="35">
+      <c r="D37" s="34">
         <f>'HOLERITE AGO.26'!C15</f>
         <v/>
       </c>
@@ -4500,7 +4607,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D38" s="35">
+      <c r="D38" s="34">
         <f>'HOLERITE AGO.26'!C16</f>
         <v/>
       </c>
@@ -4522,7 +4629,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D39" s="35">
+      <c r="D39" s="34">
         <f>'HOLERITE AGO.26'!C17</f>
         <v/>
       </c>
@@ -4544,7 +4651,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D40" s="35">
+      <c r="D40" s="34">
         <f>'HOLERITE AGO.26'!C18</f>
         <v/>
       </c>
@@ -4566,7 +4673,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D41" s="35">
+      <c r="D41" s="34">
         <f>'HOLERITE AGO.26'!C19</f>
         <v/>
       </c>
@@ -4588,7 +4695,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D42" s="35">
+      <c r="D42" s="34">
         <f>'HOLERITE AGO.26'!C20</f>
         <v/>
       </c>
@@ -4610,7 +4717,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D43" s="35">
+      <c r="D43" s="34">
         <f>'HOLERITE AGO.26'!C21</f>
         <v/>
       </c>
@@ -4654,7 +4761,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D45" s="35">
+      <c r="D45" s="34">
         <f>'HOLERITE AGO.26'!C24</f>
         <v/>
       </c>
@@ -4676,7 +4783,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D46" s="35">
+      <c r="D46" s="34">
         <f>'HOLERITE AGO.26'!C25</f>
         <v/>
       </c>
@@ -4698,7 +4805,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D47" s="35">
+      <c r="D47" s="34">
         <f>'HOLERITE AGO.26'!C26</f>
         <v/>
       </c>
@@ -4720,7 +4827,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D48" s="35">
+      <c r="D48" s="34">
         <f>'HOLERITE AGO.26'!C27</f>
         <v/>
       </c>
@@ -4742,7 +4849,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D49" s="35">
+      <c r="D49" s="34">
         <f>'HOLERITE AGO.26'!C28</f>
         <v/>
       </c>
@@ -4764,7 +4871,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D50" s="35">
+      <c r="D50" s="34">
         <f>'HOLERITE AGO.26'!C29</f>
         <v/>
       </c>
@@ -4786,7 +4893,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D51" s="35">
+      <c r="D51" s="34">
         <f>'HOLERITE AGO.26'!C30</f>
         <v/>
       </c>
@@ -4852,7 +4959,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D55" s="35">
+      <c r="D55" s="34">
         <f>'HOLERITE AGO.26'!D6</f>
         <v/>
       </c>
@@ -4874,7 +4981,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D56" s="35">
+      <c r="D56" s="34">
         <f>'HOLERITE AGO.26'!D7</f>
         <v/>
       </c>
@@ -4896,7 +5003,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D57" s="35">
+      <c r="D57" s="34">
         <f>'HOLERITE AGO.26'!D8</f>
         <v/>
       </c>
@@ -4918,7 +5025,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D58" s="35">
+      <c r="D58" s="34">
         <f>'HOLERITE AGO.26'!D11</f>
         <v/>
       </c>
@@ -4940,7 +5047,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D59" s="35">
+      <c r="D59" s="34">
         <f>'HOLERITE AGO.26'!D12</f>
         <v/>
       </c>
@@ -4962,7 +5069,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D60" s="35">
+      <c r="D60" s="34">
         <f>'HOLERITE AGO.26'!D13</f>
         <v/>
       </c>
@@ -4984,7 +5091,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D61" s="35">
+      <c r="D61" s="34">
         <f>'HOLERITE AGO.26'!D14</f>
         <v/>
       </c>
@@ -5006,7 +5113,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D62" s="35">
+      <c r="D62" s="34">
         <f>'HOLERITE AGO.26'!D15</f>
         <v/>
       </c>
@@ -5028,7 +5135,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D63" s="35">
+      <c r="D63" s="34">
         <f>'HOLERITE AGO.26'!D16</f>
         <v/>
       </c>
@@ -5050,7 +5157,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D64" s="35">
+      <c r="D64" s="34">
         <f>'HOLERITE AGO.26'!D17</f>
         <v/>
       </c>
@@ -5072,7 +5179,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D65" s="35">
+      <c r="D65" s="34">
         <f>'HOLERITE AGO.26'!D18</f>
         <v/>
       </c>
@@ -5094,7 +5201,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D66" s="35">
+      <c r="D66" s="34">
         <f>'HOLERITE AGO.26'!D19</f>
         <v/>
       </c>
@@ -5116,7 +5223,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D67" s="35">
+      <c r="D67" s="34">
         <f>'HOLERITE AGO.26'!D20</f>
         <v/>
       </c>
@@ -5138,7 +5245,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D68" s="35">
+      <c r="D68" s="34">
         <f>'HOLERITE AGO.26'!D21</f>
         <v/>
       </c>
@@ -5182,7 +5289,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D70" s="35">
+      <c r="D70" s="34">
         <f>'HOLERITE AGO.26'!D24</f>
         <v/>
       </c>
@@ -5204,7 +5311,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D71" s="35">
+      <c r="D71" s="34">
         <f>'HOLERITE AGO.26'!D25</f>
         <v/>
       </c>
@@ -5226,7 +5333,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D72" s="35">
+      <c r="D72" s="34">
         <f>'HOLERITE AGO.26'!D26</f>
         <v/>
       </c>
@@ -5248,7 +5355,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D73" s="35">
+      <c r="D73" s="34">
         <f>'HOLERITE AGO.26'!D27</f>
         <v/>
       </c>
@@ -5270,7 +5377,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D74" s="35">
+      <c r="D74" s="34">
         <f>'HOLERITE AGO.26'!D28</f>
         <v/>
       </c>
@@ -5292,7 +5399,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D75" s="35">
+      <c r="D75" s="34">
         <f>'HOLERITE AGO.26'!D29</f>
         <v/>
       </c>
@@ -5314,7 +5421,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D76" s="35">
+      <c r="D76" s="34">
         <f>'HOLERITE AGO.26'!D30</f>
         <v/>
       </c>
@@ -5380,7 +5487,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D80" s="35">
+      <c r="D80" s="34">
         <f>'HOLERITE AGO.26'!E6</f>
         <v/>
       </c>
@@ -5402,7 +5509,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D81" s="35">
+      <c r="D81" s="34">
         <f>'HOLERITE AGO.26'!E7</f>
         <v/>
       </c>
@@ -5424,7 +5531,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D82" s="35">
+      <c r="D82" s="34">
         <f>'HOLERITE AGO.26'!E8</f>
         <v/>
       </c>
@@ -5446,7 +5553,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D83" s="35">
+      <c r="D83" s="34">
         <f>'HOLERITE AGO.26'!E11</f>
         <v/>
       </c>
@@ -5468,7 +5575,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D84" s="35">
+      <c r="D84" s="34">
         <f>'HOLERITE AGO.26'!E12</f>
         <v/>
       </c>
@@ -5490,7 +5597,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D85" s="35">
+      <c r="D85" s="34">
         <f>'HOLERITE AGO.26'!E13</f>
         <v/>
       </c>
@@ -5512,7 +5619,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D86" s="35">
+      <c r="D86" s="34">
         <f>'HOLERITE AGO.26'!E14</f>
         <v/>
       </c>
@@ -5534,7 +5641,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D87" s="35">
+      <c r="D87" s="34">
         <f>'HOLERITE AGO.26'!E15</f>
         <v/>
       </c>
@@ -5556,7 +5663,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D88" s="35">
+      <c r="D88" s="34">
         <f>'HOLERITE AGO.26'!E16</f>
         <v/>
       </c>
@@ -5578,7 +5685,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D89" s="35">
+      <c r="D89" s="34">
         <f>'HOLERITE AGO.26'!E17</f>
         <v/>
       </c>
@@ -5600,7 +5707,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D90" s="35">
+      <c r="D90" s="34">
         <f>'HOLERITE AGO.26'!E18</f>
         <v/>
       </c>
@@ -5622,7 +5729,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D91" s="35">
+      <c r="D91" s="34">
         <f>'HOLERITE AGO.26'!E19</f>
         <v/>
       </c>
@@ -5644,7 +5751,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D92" s="35">
+      <c r="D92" s="34">
         <f>'HOLERITE AGO.26'!E20</f>
         <v/>
       </c>
@@ -5666,7 +5773,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D93" s="35">
+      <c r="D93" s="34">
         <f>'HOLERITE AGO.26'!E21</f>
         <v/>
       </c>
@@ -5710,7 +5817,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D95" s="35">
+      <c r="D95" s="34">
         <f>'HOLERITE AGO.26'!E24</f>
         <v/>
       </c>
@@ -5732,7 +5839,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D96" s="35">
+      <c r="D96" s="34">
         <f>'HOLERITE AGO.26'!E25</f>
         <v/>
       </c>
@@ -5754,7 +5861,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D97" s="35">
+      <c r="D97" s="34">
         <f>'HOLERITE AGO.26'!E26</f>
         <v/>
       </c>
@@ -5776,7 +5883,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D98" s="35">
+      <c r="D98" s="34">
         <f>'HOLERITE AGO.26'!E27</f>
         <v/>
       </c>
@@ -5798,7 +5905,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D99" s="35">
+      <c r="D99" s="34">
         <f>'HOLERITE AGO.26'!E28</f>
         <v/>
       </c>
@@ -5820,7 +5927,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D100" s="35">
+      <c r="D100" s="34">
         <f>'HOLERITE AGO.26'!E29</f>
         <v/>
       </c>
@@ -5842,7 +5949,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D101" s="35">
+      <c r="D101" s="34">
         <f>'HOLERITE AGO.26'!E30</f>
         <v/>
       </c>
@@ -5908,7 +6015,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D105" s="35">
+      <c r="D105" s="34">
         <f>'HOLERITE AGO.26'!F6</f>
         <v/>
       </c>
@@ -5930,7 +6037,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D106" s="35">
+      <c r="D106" s="34">
         <f>'HOLERITE AGO.26'!F7</f>
         <v/>
       </c>
@@ -5952,7 +6059,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D107" s="35">
+      <c r="D107" s="34">
         <f>'HOLERITE AGO.26'!F8</f>
         <v/>
       </c>
@@ -5974,7 +6081,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D108" s="35">
+      <c r="D108" s="34">
         <f>'HOLERITE AGO.26'!F11</f>
         <v/>
       </c>
@@ -5996,7 +6103,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D109" s="35">
+      <c r="D109" s="34">
         <f>'HOLERITE AGO.26'!F12</f>
         <v/>
       </c>
@@ -6018,7 +6125,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D110" s="35">
+      <c r="D110" s="34">
         <f>'HOLERITE AGO.26'!F13</f>
         <v/>
       </c>
@@ -6040,7 +6147,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D111" s="35">
+      <c r="D111" s="34">
         <f>'HOLERITE AGO.26'!F14</f>
         <v/>
       </c>
@@ -6062,7 +6169,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D112" s="35">
+      <c r="D112" s="34">
         <f>'HOLERITE AGO.26'!F15</f>
         <v/>
       </c>
@@ -6084,7 +6191,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D113" s="35">
+      <c r="D113" s="34">
         <f>'HOLERITE AGO.26'!F16</f>
         <v/>
       </c>
@@ -6106,7 +6213,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D114" s="35">
+      <c r="D114" s="34">
         <f>'HOLERITE AGO.26'!F17</f>
         <v/>
       </c>
@@ -6128,7 +6235,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D115" s="35">
+      <c r="D115" s="34">
         <f>'HOLERITE AGO.26'!F18</f>
         <v/>
       </c>
@@ -6150,7 +6257,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D116" s="35">
+      <c r="D116" s="34">
         <f>'HOLERITE AGO.26'!F19</f>
         <v/>
       </c>
@@ -6172,7 +6279,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D117" s="35">
+      <c r="D117" s="34">
         <f>'HOLERITE AGO.26'!F20</f>
         <v/>
       </c>
@@ -6194,7 +6301,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D118" s="35">
+      <c r="D118" s="34">
         <f>'HOLERITE AGO.26'!F21</f>
         <v/>
       </c>
@@ -6238,7 +6345,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D120" s="35">
+      <c r="D120" s="34">
         <f>'HOLERITE AGO.26'!F24</f>
         <v/>
       </c>
@@ -6260,7 +6367,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D121" s="35">
+      <c r="D121" s="34">
         <f>'HOLERITE AGO.26'!F25</f>
         <v/>
       </c>
@@ -6282,7 +6389,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D122" s="35">
+      <c r="D122" s="34">
         <f>'HOLERITE AGO.26'!F26</f>
         <v/>
       </c>
@@ -6304,7 +6411,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D123" s="35">
+      <c r="D123" s="34">
         <f>'HOLERITE AGO.26'!F27</f>
         <v/>
       </c>
@@ -6326,7 +6433,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D124" s="35">
+      <c r="D124" s="34">
         <f>'HOLERITE AGO.26'!F28</f>
         <v/>
       </c>
@@ -6348,7 +6455,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D125" s="35">
+      <c r="D125" s="34">
         <f>'HOLERITE AGO.26'!F29</f>
         <v/>
       </c>
@@ -6370,7 +6477,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D126" s="35">
+      <c r="D126" s="34">
         <f>'HOLERITE AGO.26'!F30</f>
         <v/>
       </c>
@@ -6436,7 +6543,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D130" s="35">
+      <c r="D130" s="34">
         <f>'HOLERITE AGO.26'!G6</f>
         <v/>
       </c>
@@ -6458,7 +6565,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D131" s="35">
+      <c r="D131" s="34">
         <f>'HOLERITE AGO.26'!G7</f>
         <v/>
       </c>
@@ -6480,7 +6587,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D132" s="35">
+      <c r="D132" s="34">
         <f>'HOLERITE AGO.26'!G8</f>
         <v/>
       </c>
@@ -6502,7 +6609,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D133" s="35">
+      <c r="D133" s="34">
         <f>'HOLERITE AGO.26'!G11</f>
         <v/>
       </c>
@@ -6524,7 +6631,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D134" s="35">
+      <c r="D134" s="34">
         <f>'HOLERITE AGO.26'!G12</f>
         <v/>
       </c>
@@ -6546,7 +6653,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D135" s="35">
+      <c r="D135" s="34">
         <f>'HOLERITE AGO.26'!G13</f>
         <v/>
       </c>
@@ -6568,7 +6675,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D136" s="35">
+      <c r="D136" s="34">
         <f>'HOLERITE AGO.26'!G14</f>
         <v/>
       </c>
@@ -6590,7 +6697,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D137" s="35">
+      <c r="D137" s="34">
         <f>'HOLERITE AGO.26'!G15</f>
         <v/>
       </c>
@@ -6612,7 +6719,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D138" s="35">
+      <c r="D138" s="34">
         <f>'HOLERITE AGO.26'!G16</f>
         <v/>
       </c>
@@ -6634,7 +6741,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D139" s="35">
+      <c r="D139" s="34">
         <f>'HOLERITE AGO.26'!G17</f>
         <v/>
       </c>
@@ -6656,7 +6763,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D140" s="35">
+      <c r="D140" s="34">
         <f>'HOLERITE AGO.26'!G18</f>
         <v/>
       </c>
@@ -6678,7 +6785,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D141" s="35">
+      <c r="D141" s="34">
         <f>'HOLERITE AGO.26'!G19</f>
         <v/>
       </c>
@@ -6700,7 +6807,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D142" s="35">
+      <c r="D142" s="34">
         <f>'HOLERITE AGO.26'!G20</f>
         <v/>
       </c>
@@ -6722,7 +6829,7 @@
           <t>Provento</t>
         </is>
       </c>
-      <c r="D143" s="35">
+      <c r="D143" s="34">
         <f>'HOLERITE AGO.26'!G21</f>
         <v/>
       </c>
@@ -6766,7 +6873,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D145" s="35">
+      <c r="D145" s="34">
         <f>'HOLERITE AGO.26'!G24</f>
         <v/>
       </c>
@@ -6788,7 +6895,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D146" s="35">
+      <c r="D146" s="34">
         <f>'HOLERITE AGO.26'!G25</f>
         <v/>
       </c>
@@ -6810,7 +6917,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D147" s="35">
+      <c r="D147" s="34">
         <f>'HOLERITE AGO.26'!G26</f>
         <v/>
       </c>
@@ -6832,7 +6939,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D148" s="35">
+      <c r="D148" s="34">
         <f>'HOLERITE AGO.26'!G27</f>
         <v/>
       </c>
@@ -6854,7 +6961,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D149" s="35">
+      <c r="D149" s="34">
         <f>'HOLERITE AGO.26'!G28</f>
         <v/>
       </c>
@@ -6876,7 +6983,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D150" s="35">
+      <c r="D150" s="34">
         <f>'HOLERITE AGO.26'!G29</f>
         <v/>
       </c>
@@ -6898,7 +7005,7 @@
           <t>Desconto</t>
         </is>
       </c>
-      <c r="D151" s="35">
+      <c r="D151" s="34">
         <f>'HOLERITE AGO.26'!G30</f>
         <v/>
       </c>
@@ -7019,7 +7126,7 @@
           <t>Salário base</t>
         </is>
       </c>
-      <c r="C7" s="35">
+      <c r="C7" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$6:$G$6,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
@@ -7030,7 +7137,7 @@
           <t>Adicional noturno</t>
         </is>
       </c>
-      <c r="C8" s="35">
+      <c r="C8" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$7:$G$7,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
@@ -7041,7 +7148,7 @@
           <t>Horas extras</t>
         </is>
       </c>
-      <c r="C9" s="35">
+      <c r="C9" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$8:$G$8,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
@@ -7052,7 +7159,7 @@
           <t>Comissão sobre vendas</t>
         </is>
       </c>
-      <c r="C10" s="35">
+      <c r="C10" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$11:$G$11,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
@@ -7063,7 +7170,7 @@
           <t>Repouso remunerado / DSR</t>
         </is>
       </c>
-      <c r="C11" s="35">
+      <c r="C11" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$12:$G$12,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
@@ -7074,7 +7181,7 @@
           <t>Auxílio gerência</t>
         </is>
       </c>
-      <c r="C12" s="35">
+      <c r="C12" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$13:$G$13,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
@@ -7085,7 +7192,7 @@
           <t>Adicional prêmio meta caixa</t>
         </is>
       </c>
-      <c r="C13" s="35">
+      <c r="C13" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$14:$G$14,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
@@ -7096,7 +7203,7 @@
           <t>Prêmio cota geral</t>
         </is>
       </c>
-      <c r="C14" s="35">
+      <c r="C14" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$15:$G$15,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
@@ -7107,7 +7214,7 @@
           <t>Prêmio pré-vencidos</t>
         </is>
       </c>
-      <c r="C15" s="35">
+      <c r="C15" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$16:$G$16,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
@@ -7118,7 +7225,7 @@
           <t>Férias</t>
         </is>
       </c>
-      <c r="C16" s="35">
+      <c r="C16" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$17:$G$17,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
@@ -7129,7 +7236,7 @@
           <t>1/3 constitucional de férias</t>
         </is>
       </c>
-      <c r="C17" s="35">
+      <c r="C17" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$18:$G$18,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
@@ -7140,7 +7247,7 @@
           <t>Incentivo aplicações</t>
         </is>
       </c>
-      <c r="C18" s="35">
+      <c r="C18" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$19:$G$19,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
@@ -7151,7 +7258,7 @@
           <t>Incentivo vitaminas</t>
         </is>
       </c>
-      <c r="C19" s="35">
+      <c r="C19" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$20:$G$20,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
@@ -7162,7 +7269,7 @@
           <t>Outros incentivos</t>
         </is>
       </c>
-      <c r="C20" s="35">
+      <c r="C20" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$21:$G$21,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
@@ -7193,7 +7300,7 @@
           <t>Adiantamento / vales</t>
         </is>
       </c>
-      <c r="C23" s="35">
+      <c r="C23" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$24:$G$24,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
@@ -7204,7 +7311,7 @@
           <t>Adiantamento de incentivos e aplicações</t>
         </is>
       </c>
-      <c r="C24" s="35">
+      <c r="C24" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$25:$G$25,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
@@ -7215,7 +7322,7 @@
           <t>Convênio</t>
         </is>
       </c>
-      <c r="C25" s="35">
+      <c r="C25" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$26:$G$26,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
@@ -7226,7 +7333,7 @@
           <t>Faltas / atrasos</t>
         </is>
       </c>
-      <c r="C26" s="35">
+      <c r="C26" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$27:$G$27,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
@@ -7237,7 +7344,7 @@
           <t>Vale transporte 6%</t>
         </is>
       </c>
-      <c r="C27" s="35">
+      <c r="C27" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$28:$G$28,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
@@ -7248,7 +7355,7 @@
           <t>INSS</t>
         </is>
       </c>
-      <c r="C28" s="35">
+      <c r="C28" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$29:$G$29,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
@@ -7259,7 +7366,7 @@
           <t>IRRF</t>
         </is>
       </c>
-      <c r="C29" s="35">
+      <c r="C29" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$30:$G$30,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
@@ -7308,7 +7415,7 @@
           <t>Venda bruta</t>
         </is>
       </c>
-      <c r="C35" s="35">
+      <c r="C35" s="34">
         <f>IFERROR(INDEX('BASE INOVAFARMA AGO.26'!$C$5:$C$10,MATCH($C$4,'BASE INOVAFARMA AGO.26'!$B$5:$B$10,0)),0)</f>
         <v/>
       </c>
@@ -7319,7 +7426,7 @@
           <t>Descontos concedidos</t>
         </is>
       </c>
-      <c r="C36" s="35">
+      <c r="C36" s="34">
         <f>IFERROR(INDEX('BASE INOVAFARMA AGO.26'!$D$5:$D$10,MATCH($C$4,'BASE INOVAFARMA AGO.26'!$B$5:$B$10,0)),0)</f>
         <v/>
       </c>
@@ -7330,7 +7437,7 @@
           <t>Venda líquida</t>
         </is>
       </c>
-      <c r="C37" s="35">
+      <c r="C37" s="34">
         <f>IFERROR(INDEX('BASE INOVAFARMA AGO.26'!$E$5:$E$10,MATCH($C$4,'BASE INOVAFARMA AGO.26'!$B$5:$B$10,0)),0)</f>
         <v/>
       </c>
@@ -7341,7 +7448,7 @@
           <t>Comissão apurada</t>
         </is>
       </c>
-      <c r="C38" s="35">
+      <c r="C38" s="34">
         <f>IFERROR(INDEX('BASE INOVAFARMA AGO.26'!$F$5:$F$10,MATCH($C$4,'BASE INOVAFARMA AGO.26'!$B$5:$B$10,0)),0)</f>
         <v/>
       </c>
@@ -7352,7 +7459,7 @@
           <t>Total de incentivos</t>
         </is>
       </c>
-      <c r="C39" s="35">
+      <c r="C39" s="34">
         <f>IFERROR(INDEX('BASE INOVAFARMA AGO.26'!$J$5:$J$10,MATCH($C$4,'BASE INOVAFARMA AGO.26'!$B$5:$B$10,0)),0)</f>
         <v/>
       </c>
@@ -7399,6 +7506,283 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="62" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>APONTAMENTO DO PONTO — AGOSTO/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Loja CENTRO · horas extras, adicional noturno e feriado trabalhado · alimenta a aba HOLERITE AGO.26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>FUNCIONÁRIO</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>OCORRÊNCIA</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>QTDE</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>UNIDADE</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>SALÁRIO BASE</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>VALOR UNITÁRIO</t>
+        </is>
+      </c>
+      <c r="G4" s="13" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="H4" s="13" t="inlineStr">
+        <is>
+          <t>RUBRICA DESTINO</t>
+        </is>
+      </c>
+      <c r="I4" s="13" t="inlineStr">
+        <is>
+          <t>OBSERVAÇÃO</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="53" t="n"/>
+      <c r="B5" s="53" t="n"/>
+      <c r="C5" s="53" t="n"/>
+      <c r="D5" s="53" t="n"/>
+      <c r="E5" s="34">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$6:$G$6,1,MATCH(A5,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
+        <v/>
+      </c>
+      <c r="F5" s="35" t="n"/>
+      <c r="G5" s="20">
+        <f>ROUND(C5*F5,2)</f>
+        <v/>
+      </c>
+      <c r="H5" s="53" t="n"/>
+      <c r="I5" s="53" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="53" t="n"/>
+      <c r="B6" s="53" t="n"/>
+      <c r="C6" s="53" t="n"/>
+      <c r="D6" s="53" t="n"/>
+      <c r="E6" s="34">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$6:$G$6,1,MATCH(A6,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
+        <v/>
+      </c>
+      <c r="F6" s="35" t="n"/>
+      <c r="G6" s="20">
+        <f>ROUND(C6*F6,2)</f>
+        <v/>
+      </c>
+      <c r="H6" s="53" t="n"/>
+      <c r="I6" s="53" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="53" t="n"/>
+      <c r="B7" s="53" t="n"/>
+      <c r="C7" s="53" t="n"/>
+      <c r="D7" s="53" t="n"/>
+      <c r="E7" s="34">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$6:$G$6,1,MATCH(A7,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
+        <v/>
+      </c>
+      <c r="F7" s="35" t="n"/>
+      <c r="G7" s="20">
+        <f>ROUND(C7*F7,2)</f>
+        <v/>
+      </c>
+      <c r="H7" s="53" t="n"/>
+      <c r="I7" s="53" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="53" t="n"/>
+      <c r="B8" s="53" t="n"/>
+      <c r="C8" s="53" t="n"/>
+      <c r="D8" s="53" t="n"/>
+      <c r="E8" s="34">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$6:$G$6,1,MATCH(A8,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
+        <v/>
+      </c>
+      <c r="F8" s="35" t="n"/>
+      <c r="G8" s="20">
+        <f>ROUND(C8*F8,2)</f>
+        <v/>
+      </c>
+      <c r="H8" s="53" t="n"/>
+      <c r="I8" s="53" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="53" t="n"/>
+      <c r="B9" s="53" t="n"/>
+      <c r="C9" s="53" t="n"/>
+      <c r="D9" s="53" t="n"/>
+      <c r="E9" s="34">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$6:$G$6,1,MATCH(A9,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
+        <v/>
+      </c>
+      <c r="F9" s="35" t="n"/>
+      <c r="G9" s="20">
+        <f>ROUND(C9*F9,2)</f>
+        <v/>
+      </c>
+      <c r="H9" s="53" t="n"/>
+      <c r="I9" s="53" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="53" t="n"/>
+      <c r="B10" s="53" t="n"/>
+      <c r="C10" s="53" t="n"/>
+      <c r="D10" s="53" t="n"/>
+      <c r="E10" s="34">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$6:$G$6,1,MATCH(A10,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
+        <v/>
+      </c>
+      <c r="F10" s="35" t="n"/>
+      <c r="G10" s="20">
+        <f>ROUND(C10*F10,2)</f>
+        <v/>
+      </c>
+      <c r="H10" s="53" t="n"/>
+      <c r="I10" s="53" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="53" t="n"/>
+      <c r="B11" s="53" t="n"/>
+      <c r="C11" s="53" t="n"/>
+      <c r="D11" s="53" t="n"/>
+      <c r="E11" s="34">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$6:$G$6,1,MATCH(A11,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
+        <v/>
+      </c>
+      <c r="F11" s="35" t="n"/>
+      <c r="G11" s="20">
+        <f>ROUND(C11*F11,2)</f>
+        <v/>
+      </c>
+      <c r="H11" s="53" t="n"/>
+      <c r="I11" s="53" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="53" t="n"/>
+      <c r="B12" s="53" t="n"/>
+      <c r="C12" s="53" t="n"/>
+      <c r="D12" s="53" t="n"/>
+      <c r="E12" s="34">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$6:$G$6,1,MATCH(A12,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
+        <v/>
+      </c>
+      <c r="F12" s="35" t="n"/>
+      <c r="G12" s="20">
+        <f>ROUND(C12*F12,2)</f>
+        <v/>
+      </c>
+      <c r="H12" s="53" t="n"/>
+      <c r="I12" s="53" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="18" t="n"/>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="n"/>
+      <c r="D13" s="18" t="n"/>
+      <c r="E13" s="18" t="n"/>
+      <c r="F13" s="18" t="n"/>
+      <c r="G13" s="20">
+        <f>SUM(G5:G12)</f>
+        <v/>
+      </c>
+      <c r="H13" s="18" t="n"/>
+      <c r="I13" s="18" t="n"/>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>Salário-hora = salário base ÷ 220. Hora extra = salário-hora × 1,5. Adicional noturno = salário-hora × 20%. Feriado trabalhado sem folga = 1 salário-dia a mais (salário base ÷ 30).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>No salário de R$ 1.621,00: 40 horas extras dão R$ 442,09 e 24 horas dão R$ 265,25 — é a mesma conta usada na planilha de julho.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>As linhas em branco são para acrescentar ocorrências: preencha funcionário, ocorrência, quantidade, valor unitário e a rubrica de destino (HORAS EXTRAS ou ADICIONAL NOTURNO).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>Os totais desta aba entram sozinhos nas linhas HORAS EXTRAS e ADICIONAL NOTURNO da aba HOLERITE AGO.26.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:I12"/>
+  <mergeCells count="6">
+    <mergeCell ref="A15:I15"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A18:I18"/>
+    <mergeCell ref="A16:I16"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -7479,18 +7863,18 @@
           <t>51</t>
         </is>
       </c>
-      <c r="C5" s="34" t="n">
+      <c r="C5" s="35" t="n">
         <v>150</v>
       </c>
       <c r="D5" s="8" t="n"/>
-      <c r="E5" s="53">
+      <c r="E5" s="54">
         <f>C5*D5</f>
         <v/>
       </c>
-      <c r="F5" s="34" t="n">
+      <c r="F5" s="35" t="n">
         <v>128.8</v>
       </c>
-      <c r="G5" s="34" t="n">
+      <c r="G5" s="35" t="n">
         <v>40</v>
       </c>
       <c r="H5" s="38">
@@ -7509,18 +7893,18 @@
           <t>131</t>
         </is>
       </c>
-      <c r="C6" s="34" t="n">
+      <c r="C6" s="35" t="n">
         <v>100</v>
       </c>
       <c r="D6" s="8" t="n"/>
-      <c r="E6" s="53">
+      <c r="E6" s="54">
         <f>C6*D6</f>
         <v/>
       </c>
-      <c r="F6" s="34" t="n">
+      <c r="F6" s="35" t="n">
         <v>83.56</v>
       </c>
-      <c r="G6" s="34" t="n">
+      <c r="G6" s="35" t="n">
         <v>0</v>
       </c>
       <c r="H6" s="38">

</xml_diff>

<commit_message>
Corrigir rótulos lidos como fórmula e somar as horas extras da NATI
- Textos que começavam com "=" viravam #ERROR! no Google Planilhas: o
  rótulo da linha de comissão total e a observação do DSR
- NATI: as 17 horas noturnas eram horas extras — passam a gerar a hora
  extra de 50% (R$ 187,89) além do adicional noturno (R$ 25,05)
- GENECIR: sem desconto de vale-transporte, já que passou agosto inteiro
  de férias
- Novo resumo consolidado das três lojas para enviar à contabilidade

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2n4hj3F39Ez9XRrPSJYG5
</commit_message>
<xml_diff>
--- a/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_CENTRO_pgto_05-09-2026.xlsx
+++ b/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_CENTRO_pgto_05-09-2026.xlsx
@@ -2139,9 +2139,10 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15">
-        <f> COMISSÃO TOTAL</f>
-        <v/>
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>COMISSÃO TOTAL (soma)</t>
+        </is>
       </c>
       <c r="B11" s="20">
         <f>SUM(B9:B10)</f>
@@ -2211,9 +2212,10 @@
         <f>SUM(B12:G12)</f>
         <v/>
       </c>
-      <c r="I12" s="33">
-        <f> (comissão total + horas extras) × 5 domingos ÷ 26 dias úteis de agosto/2026.</f>
-        <v/>
+      <c r="I12" s="33" t="inlineStr">
+        <is>
+          <t>Cálculo: (comissão total + horas extras) × 5 domingos ÷ 26 dias úteis de agosto/2026.</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -2639,9 +2641,7 @@
       <c r="C28" s="31" t="n">
         <v>-84.29000000000001</v>
       </c>
-      <c r="D28" s="31" t="n">
-        <v>-84.29000000000001</v>
-      </c>
+      <c r="D28" s="31" t="n"/>
       <c r="E28" s="31" t="n">
         <v>-74.29000000000001</v>
       </c>
@@ -2655,7 +2655,7 @@
       </c>
       <c r="I28" s="33" t="inlineStr">
         <is>
-          <t>Valores praticados em jul/26. 6% sobre R$ 1.621,00 seria R$ 97,26 — CONFERIR a base usada.</t>
+          <t>Valores praticados em jul/26. 6% sobre R$ 1.621,00 seria R$ 97,26 — CONFERIR a base usada. Quem passou o mês em férias fica sem desconto.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Incluir adiantamento salarial e férias à parte nas três lojas
- A rubrica de vales passa a se chamar ADIANTAMENTO SALARIAL / VALES,
  igual ao resumo
- Nova linha FÉRIAS PAGAS À PARTE (CONTAS A PAGAR) no bloco informativo,
  fora do líquido, com a observação de quem teve férias no mês
- Setembro: RENALDO (Centro) e VALDICK (Trancoso) de férias de 01 a
  30/09 — salário zerado, sem desconto de vale-transporte e registro na
  aba de ponto

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2n4hj3F39Ez9XRrPSJYG5
</commit_message>
<xml_diff>
--- a/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_CENTRO_pgto_05-09-2026.xlsx
+++ b/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_CENTRO_pgto_05-09-2026.xlsx
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'BASE INOVAFARMA AGO.26'!$A$4:$J$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'HOLERITE AGO.26'!$A$4:$I$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'HOLERITE AGO.26'!$A$4:$I$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'JULHO.26 REVISADO'!$A$4:$I$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'LISTA CONTABILIDADE'!$A$4:$E$153</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="6">'GANHOS DO COLABORADOR'!$A$1:$D$44</definedName>
@@ -1874,7 +1874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2528,7 +2528,7 @@
     <row r="24">
       <c r="A24" s="30" t="inlineStr">
         <is>
-          <t>ADIANTAMENTO / VALES</t>
+          <t>ADIANTAMENTO SALARIAL / VALES</t>
         </is>
       </c>
       <c r="B24" s="35" t="n"/>
@@ -2853,70 +2853,92 @@
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="21" t="inlineStr">
-        <is>
-          <t>LEGENDA</t>
-        </is>
-      </c>
-      <c r="B38" s="22" t="inlineStr"/>
+    <row r="37">
+      <c r="A37" s="30" t="inlineStr">
+        <is>
+          <t>FÉRIAS PAGAS À PARTE (CONTAS A PAGAR)</t>
+        </is>
+      </c>
+      <c r="B37" s="31" t="n"/>
+      <c r="C37" s="31" t="n"/>
+      <c r="D37" s="31" t="n"/>
+      <c r="E37" s="31" t="n"/>
+      <c r="F37" s="31" t="n"/>
+      <c r="G37" s="31" t="n"/>
+      <c r="H37" s="32">
+        <f>SUM(B37:G37)</f>
+        <v/>
+      </c>
+      <c r="I37" s="33" t="inlineStr">
+        <is>
+          <t>Recibo de férias pago fora do holerite — lembrete para o contas a pagar. GENECIR: férias de 01 a 30/08/2026, pagas em recibo próprio — informar o valor.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="21" t="inlineStr">
         <is>
-          <t>Célula amarela, texto azul</t>
-        </is>
-      </c>
-      <c r="B39" s="22" t="inlineStr">
-        <is>
-          <t>valor digitado — PREENCHER ou conferir antes de enviar.</t>
-        </is>
-      </c>
+          <t>LEGENDA</t>
+        </is>
+      </c>
+      <c r="B39" s="22" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="21" t="inlineStr">
         <is>
-          <t>Célula laranja</t>
+          <t>Célula amarela, texto azul</t>
         </is>
       </c>
       <c r="B40" s="22" t="inlineStr">
         <is>
-          <t>valor repetido de julho/2026 — CONFERIR se continua válido em agosto.</t>
+          <t>valor digitado — PREENCHER ou conferir antes de enviar.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="21" t="inlineStr">
         <is>
-          <t>Texto verde</t>
+          <t>Célula laranja</t>
         </is>
       </c>
       <c r="B41" s="22" t="inlineStr">
         <is>
-          <t>valor puxado da aba BASE INOVAFARMA AGO.26 (não digitar por cima).</t>
+          <t>valor repetido de julho/2026 — CONFERIR se continua válido em agosto.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="21" t="inlineStr">
         <is>
+          <t>Texto verde</t>
+        </is>
+      </c>
+      <c r="B42" s="22" t="inlineStr">
+        <is>
+          <t>valor puxado da aba BASE INOVAFARMA AGO.26 (não digitar por cima).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="21" t="inlineStr">
+        <is>
           <t>Texto preto em célula verde</t>
         </is>
       </c>
-      <c r="B42" s="22" t="inlineStr">
+      <c r="B43" s="22" t="inlineStr">
         <is>
           <t>resultado de fórmula — não alterar.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I36"/>
+  <autoFilter ref="A4:I37"/>
   <mergeCells count="7">
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="B39:I39"/>
-    <mergeCell ref="B38:I38"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="B42:I42"/>
+    <mergeCell ref="B43:I43"/>
     <mergeCell ref="B41:I41"/>
     <mergeCell ref="B40:I40"/>
   </mergeCells>
@@ -4225,7 +4247,7 @@
       </c>
       <c r="B20" s="30" t="inlineStr">
         <is>
-          <t>ADIANTAMENTO / VALES</t>
+          <t>ADIANTAMENTO SALARIAL / VALES</t>
         </is>
       </c>
       <c r="C20" s="30" t="inlineStr">
@@ -4753,7 +4775,7 @@
       </c>
       <c r="B45" s="30" t="inlineStr">
         <is>
-          <t>ADIANTAMENTO / VALES</t>
+          <t>ADIANTAMENTO SALARIAL / VALES</t>
         </is>
       </c>
       <c r="C45" s="30" t="inlineStr">
@@ -5281,7 +5303,7 @@
       </c>
       <c r="B70" s="30" t="inlineStr">
         <is>
-          <t>ADIANTAMENTO / VALES</t>
+          <t>ADIANTAMENTO SALARIAL / VALES</t>
         </is>
       </c>
       <c r="C70" s="30" t="inlineStr">
@@ -5809,7 +5831,7 @@
       </c>
       <c r="B95" s="30" t="inlineStr">
         <is>
-          <t>ADIANTAMENTO / VALES</t>
+          <t>ADIANTAMENTO SALARIAL / VALES</t>
         </is>
       </c>
       <c r="C95" s="30" t="inlineStr">
@@ -6337,7 +6359,7 @@
       </c>
       <c r="B120" s="30" t="inlineStr">
         <is>
-          <t>ADIANTAMENTO / VALES</t>
+          <t>ADIANTAMENTO SALARIAL / VALES</t>
         </is>
       </c>
       <c r="C120" s="30" t="inlineStr">
@@ -6865,7 +6887,7 @@
       </c>
       <c r="B145" s="30" t="inlineStr">
         <is>
-          <t>ADIANTAMENTO / VALES</t>
+          <t>ADIANTAMENTO SALARIAL / VALES</t>
         </is>
       </c>
       <c r="C145" s="30" t="inlineStr">
@@ -7297,7 +7319,7 @@
     <row r="23">
       <c r="B23" s="30" t="inlineStr">
         <is>
-          <t>Adiantamento / vales</t>
+          <t>Adiantamento salarial / vales</t>
         </is>
       </c>
       <c r="C23" s="34">

</xml_diff>

<commit_message>
Lançar os valores do holerite da Betel nas três lojas
Leitura dos demonstrativos de agosto/2026 das três empresas e
lançamento de prêmios, DSR sobre hora extra, salário família,
insuficiência de saldo, vales, vale-transporte, INSS e IRRF.

Novas linhas: DSR SOBRE HORAS EXTRAS, SALÁRIO FAMÍLIA e INSUFICIÊNCIA DE
SALDO, mais a conferência LÍQUIDO DO HOLERITE (BETEL) e a diferença
contra o líquido calculado. Fecha em zero em 17 dos 19 funcionários.

Pontos em aberto registrados nas capas: a comissão do JOEL fora do
holerite, o PEDRO ausente da folha do Centro, a comissão residual do
GENECIR e o DSR sobre hora extra pago em duplicidade.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2n4hj3F39Ez9XRrPSJYG5
</commit_message>
<xml_diff>
--- a/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_CENTRO_pgto_05-09-2026.xlsx
+++ b/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_CENTRO_pgto_05-09-2026.xlsx
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'BASE INOVAFARMA AGO.26'!$A$4:$J$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'HOLERITE AGO.26'!$A$4:$I$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'HOLERITE AGO.26'!$A$4:$I$42</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'JULHO.26 REVISADO'!$A$4:$I$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'LISTA CONTABILIDADE'!$A$4:$E$153</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="6">'GANHOS DO COLABORADOR'!$A$1:$D$44</definedName>
@@ -182,12 +182,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6E0B4"/>
+        <fgColor rgb="00FFF0F0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF0F0"/>
+        <fgColor rgb="00C6E0B4"/>
       </patternFill>
     </fill>
   </fills>
@@ -217,7 +217,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -230,7 +230,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -285,8 +285,10 @@
     <xf numFmtId="164" fontId="12" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="11" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -296,16 +298,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="13" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="13" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="13" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="16" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="16" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -674,7 +676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B45"/>
+  <dimension ref="A1:B47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -934,7 +936,7 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>GENECIR: as férias vão até 30/08 e o mês tem 31 dias — confirmar se o dia 31/08 foi trabalhado e lançar o salário desse dia (R$ 1.621,00 ÷ 30 = R$ 54,03).</t>
+          <t>PEDRO não aparece no holerite de agosto emitido pela Betel para esta loja — verificar em qual empresa ele foi lançado.</t>
         </is>
       </c>
     </row>
@@ -946,7 +948,7 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>Preencher a quantidade de diárias de SERGIO e ANA CELIA na aba FOLGUISTAS.</t>
+          <t>GENECIR: a comissão de R$ 0,62 não entrou no holerite (ele passou o mês de férias) — conferir se vale lançar.</t>
         </is>
       </c>
     </row>
@@ -958,29 +960,38 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
+          <t>GENECIR: as férias vão até 30/08 e o mês tem 31 dias — confirmar se o dia 31/08 foi trabalhado e lançar o salário desse dia (R$ 1.621,00 ÷ 30 = R$ 54,03).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="17" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>Preencher a quantidade de diárias de SERGIO e ANA CELIA na aba FOLGUISTAS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="17" customHeight="1">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
           <t>Confirmar se os folguistas recebem a comissão apurada no código deles (SERGIO R$ 128,80 e ANA CELIA R$ 83,56) além da diária.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>OBSERVAÇÃO TÉCNICA</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="17" customHeight="1">
-      <c r="A36" s="4" t="inlineStr"/>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>As células de total e de cálculo são fórmulas. Ao abrir no Excel ou no Google Planilhas elas aparecem calculadas; em visualizadores simples podem aparecer em branco até o arquivo ser aberto.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>ABAS DO ARQUIVO</t>
+          <t>OBSERVAÇÃO TÉCNICA</t>
         </is>
       </c>
     </row>
@@ -988,15 +999,14 @@
       <c r="A38" s="4" t="inlineStr"/>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>HOLERITE AGO.26 — relatório principal da competência agosto/2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="17" customHeight="1">
-      <c r="A39" s="4" t="inlineStr"/>
-      <c r="B39" s="5" t="inlineStr">
-        <is>
-          <t>GANHOS DO COLABORADOR — demonstrativo individual, pronto para imprimir/mandar.</t>
+          <t>As células de total e de cálculo são fórmulas. Ao abrir no Excel ou no Google Planilhas elas aparecem calculadas; em visualizadores simples podem aparecer em branco até o arquivo ser aberto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>ABAS DO ARQUIVO</t>
         </is>
       </c>
     </row>
@@ -1004,7 +1014,7 @@
       <c r="A40" s="4" t="inlineStr"/>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>LISTA CONTABILIDADE — os mesmos lançamentos em formato de lista.</t>
+          <t>HOLERITE AGO.26 — relatório principal da competência agosto/2026.</t>
         </is>
       </c>
     </row>
@@ -1012,7 +1022,7 @@
       <c r="A41" s="4" t="inlineStr"/>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>BASE INOVAFARMA AGO.26 — apuração de comissões e incentivos por vendedor.</t>
+          <t>GANHOS DO COLABORADOR — demonstrativo individual, pronto para imprimir/mandar.</t>
         </is>
       </c>
     </row>
@@ -1020,7 +1030,7 @@
       <c r="A42" s="4" t="inlineStr"/>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>JULHO.26 REVISADO — a folha de julho (CENTRO 05JULHO) reorganizada e conferida.</t>
+          <t>LISTA CONTABILIDADE — os mesmos lançamentos em formato de lista.</t>
         </is>
       </c>
     </row>
@@ -1028,7 +1038,7 @@
       <c r="A43" s="4" t="inlineStr"/>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>PARÂMETROS — calendário do mês, fator do DSR e valores fixos.</t>
+          <t>BASE INOVAFARMA AGO.26 — apuração de comissões e incentivos por vendedor.</t>
         </is>
       </c>
     </row>
@@ -1036,13 +1046,29 @@
       <c r="A44" s="4" t="inlineStr"/>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>PONTO AGO.26 — horas extras, adicional noturno e feriado trabalhado; alimenta o holerite.</t>
+          <t>JULHO.26 REVISADO — a folha de julho (CENTRO 05JULHO) reorganizada e conferida.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="17" customHeight="1">
       <c r="A45" s="4" t="inlineStr"/>
       <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>PARÂMETROS — calendário do mês, fator do DSR e valores fixos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="17" customHeight="1">
+      <c r="A46" s="4" t="inlineStr"/>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>PONTO AGO.26 — horas extras, adicional noturno e feriado trabalhado; alimenta o holerite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="17" customHeight="1">
+      <c r="A47" s="4" t="inlineStr"/>
+      <c r="B47" s="5" t="inlineStr">
         <is>
           <t>FOLGUISTAS — diárias de SERGIO e ANA CELIA para o contas a pagar (fora do holerite).</t>
         </is>
@@ -1058,7 +1084,7 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A39:B39"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1874,7 +1900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2221,73 +2247,75 @@
     <row r="13">
       <c r="A13" s="30" t="inlineStr">
         <is>
-          <t>AUXÍLIO GERÊNCIA</t>
-        </is>
-      </c>
-      <c r="B13" s="35" t="n"/>
-      <c r="C13" s="35" t="n"/>
-      <c r="D13" s="35" t="n"/>
-      <c r="E13" s="35" t="n"/>
-      <c r="F13" s="35" t="n"/>
-      <c r="G13" s="35" t="n"/>
-      <c r="H13" s="20">
+          <t>DSR SOBRE HORAS EXTRAS</t>
+        </is>
+      </c>
+      <c r="B13" s="37" t="n"/>
+      <c r="C13" s="37" t="n"/>
+      <c r="D13" s="37" t="n"/>
+      <c r="E13" s="37" t="n"/>
+      <c r="F13" s="37" t="n"/>
+      <c r="G13" s="37" t="n"/>
+      <c r="H13" s="38">
         <f>SUM(B13:G13)</f>
         <v/>
       </c>
       <c r="I13" s="33" t="inlineStr">
         <is>
-          <t>Conforme acordo da loja.</t>
+          <t>Rubrica 057 do holerite da Betel. ATENÇÃO: a rubrica 420 acima já leva as horas extras na base, então este valor paga o DSR das horas extras uma segunda vez — conferir com a contabilidade.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="30" t="inlineStr">
         <is>
-          <t>ADICIONAL PRÊMIO META CAIXA</t>
-        </is>
-      </c>
-      <c r="B14" s="35" t="n"/>
-      <c r="C14" s="35" t="n"/>
-      <c r="D14" s="35" t="n"/>
-      <c r="E14" s="35" t="n"/>
-      <c r="F14" s="35" t="n"/>
-      <c r="G14" s="35" t="n"/>
-      <c r="H14" s="20">
+          <t>SALÁRIO FAMÍLIA</t>
+        </is>
+      </c>
+      <c r="B14" s="31" t="n"/>
+      <c r="C14" s="31" t="n"/>
+      <c r="D14" s="31" t="n"/>
+      <c r="E14" s="31" t="n"/>
+      <c r="F14" s="31" t="n"/>
+      <c r="G14" s="31" t="n"/>
+      <c r="H14" s="32">
         <f>SUM(B14:G14)</f>
         <v/>
       </c>
       <c r="I14" s="33" t="inlineStr">
         <is>
-          <t>Conforme apuração do caixa.</t>
+          <t>Rubrica 599 do holerite da Betel.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="30" t="inlineStr">
         <is>
-          <t>PRÊMIO COTA GERAL</t>
-        </is>
-      </c>
-      <c r="B15" s="35" t="n"/>
-      <c r="C15" s="35" t="n"/>
-      <c r="D15" s="35" t="n"/>
-      <c r="E15" s="35" t="n"/>
-      <c r="F15" s="35" t="n"/>
-      <c r="G15" s="35" t="n"/>
-      <c r="H15" s="20">
+          <t>INSUFICIÊNCIA DE SALDO</t>
+        </is>
+      </c>
+      <c r="B15" s="31" t="n"/>
+      <c r="C15" s="31" t="n"/>
+      <c r="D15" s="31" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="E15" s="31" t="n"/>
+      <c r="F15" s="31" t="n"/>
+      <c r="G15" s="31" t="n"/>
+      <c r="H15" s="32">
         <f>SUM(B15:G15)</f>
         <v/>
       </c>
       <c r="I15" s="33" t="inlineStr">
         <is>
-          <t>PREENCHER conforme a tabela de metas da loja (aba METAS da planilha original).</t>
+          <t>Rubrica 998 do holerite da Betel — contrapartida do vale-transporte de quem ficou sem saldo.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="30" t="inlineStr">
         <is>
-          <t>PRÊMIO PRÉ-VENCIDOS</t>
+          <t>AUXÍLIO GERÊNCIA</t>
         </is>
       </c>
       <c r="B16" s="35" t="n"/>
@@ -2302,14 +2330,14 @@
       </c>
       <c r="I16" s="33" t="inlineStr">
         <is>
-          <t>PREENCHER conforme a apuração de pré-vencidos de agosto.</t>
+          <t>Conforme acordo da loja.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="30" t="inlineStr">
         <is>
-          <t>FÉRIAS (DIAS GOZADOS)</t>
+          <t>ADICIONAL PRÊMIO META CAIXA</t>
         </is>
       </c>
       <c r="B17" s="35" t="n"/>
@@ -2324,180 +2352,132 @@
       </c>
       <c r="I17" s="33" t="inlineStr">
         <is>
-          <t>PREENCHER se houve férias no mês; informar o período.</t>
+          <t>Conforme apuração do caixa.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="30" t="inlineStr">
         <is>
-          <t>1/3 CONSTITUCIONAL DE FÉRIAS</t>
-        </is>
-      </c>
-      <c r="B18" s="35" t="n"/>
-      <c r="C18" s="35" t="n"/>
-      <c r="D18" s="35" t="n"/>
-      <c r="E18" s="35" t="n"/>
-      <c r="F18" s="35" t="n"/>
-      <c r="G18" s="35" t="n"/>
-      <c r="H18" s="20">
+          <t>PRÊMIO COTA GERAL / BONIFICAÇÃO</t>
+        </is>
+      </c>
+      <c r="B18" s="31" t="n"/>
+      <c r="C18" s="31" t="n">
+        <v>600</v>
+      </c>
+      <c r="D18" s="31" t="n"/>
+      <c r="E18" s="31" t="n">
+        <v>250</v>
+      </c>
+      <c r="F18" s="31" t="n">
+        <v>100</v>
+      </c>
+      <c r="G18" s="31" t="n"/>
+      <c r="H18" s="32">
         <f>SUM(B18:G18)</f>
         <v/>
       </c>
       <c r="I18" s="33" t="inlineStr">
         <is>
-          <t>Calculado pela contabilidade sobre o valor das férias.</t>
+          <t xml:space="preserve">Rubrica 011 (Bonificação/Prêmios) do holerite da Betel — já engloba cota geral e pré-vencidos. </t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="30" t="inlineStr">
         <is>
-          <t>INCENTIVO APLICAÇÕES</t>
-        </is>
-      </c>
-      <c r="B19" s="34">
-        <f>'BASE INOVAFARMA AGO.26'!G5</f>
-        <v/>
-      </c>
-      <c r="C19" s="34">
-        <f>'BASE INOVAFARMA AGO.26'!G6</f>
-        <v/>
-      </c>
-      <c r="D19" s="34">
-        <f>'BASE INOVAFARMA AGO.26'!G7</f>
-        <v/>
-      </c>
-      <c r="E19" s="34">
-        <f>'BASE INOVAFARMA AGO.26'!G8</f>
-        <v/>
-      </c>
-      <c r="F19" s="34">
-        <f>'BASE INOVAFARMA AGO.26'!G9</f>
-        <v/>
-      </c>
-      <c r="G19" s="34">
-        <f>'BASE INOVAFARMA AGO.26'!G10</f>
-        <v/>
-      </c>
+          <t>PRÊMIO PRÉ-VENCIDOS</t>
+        </is>
+      </c>
+      <c r="B19" s="35" t="n"/>
+      <c r="C19" s="35" t="n"/>
+      <c r="D19" s="35" t="n"/>
+      <c r="E19" s="35" t="n"/>
+      <c r="F19" s="35" t="n"/>
+      <c r="G19" s="35" t="n"/>
       <c r="H19" s="20">
         <f>SUM(B19:G19)</f>
         <v/>
       </c>
       <c r="I19" s="33" t="inlineStr">
         <is>
-          <t>Incentivo de injetáveis apurado no InovaFarma.</t>
+          <t>Vem somado na linha acima, na rubrica 011 do holerite.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="30" t="inlineStr">
         <is>
-          <t>INCENTIVO VITAMINAS</t>
-        </is>
-      </c>
-      <c r="B20" s="34">
-        <f>'BASE INOVAFARMA AGO.26'!H5</f>
-        <v/>
-      </c>
-      <c r="C20" s="34">
-        <f>'BASE INOVAFARMA AGO.26'!H6</f>
-        <v/>
-      </c>
-      <c r="D20" s="34">
-        <f>'BASE INOVAFARMA AGO.26'!H7</f>
-        <v/>
-      </c>
-      <c r="E20" s="34">
-        <f>'BASE INOVAFARMA AGO.26'!H8</f>
-        <v/>
-      </c>
-      <c r="F20" s="34">
-        <f>'BASE INOVAFARMA AGO.26'!H9</f>
-        <v/>
-      </c>
-      <c r="G20" s="34">
-        <f>'BASE INOVAFARMA AGO.26'!H10</f>
-        <v/>
-      </c>
+          <t>FÉRIAS (DIAS GOZADOS)</t>
+        </is>
+      </c>
+      <c r="B20" s="35" t="n"/>
+      <c r="C20" s="35" t="n"/>
+      <c r="D20" s="35" t="n"/>
+      <c r="E20" s="35" t="n"/>
+      <c r="F20" s="35" t="n"/>
+      <c r="G20" s="35" t="n"/>
       <c r="H20" s="20">
         <f>SUM(B20:G20)</f>
         <v/>
       </c>
       <c r="I20" s="33" t="inlineStr">
         <is>
-          <t>Grupo APLICAÇÃO E VITAMINAS INCENTIVO no InovaFarma.</t>
+          <t>PREENCHER se houve férias no mês; informar o período.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="30" t="inlineStr">
         <is>
-          <t>OUTROS INCENTIVOS</t>
-        </is>
-      </c>
-      <c r="B21" s="34">
-        <f>'BASE INOVAFARMA AGO.26'!I5</f>
-        <v/>
-      </c>
-      <c r="C21" s="34">
-        <f>'BASE INOVAFARMA AGO.26'!I6</f>
-        <v/>
-      </c>
-      <c r="D21" s="34">
-        <f>'BASE INOVAFARMA AGO.26'!I7</f>
-        <v/>
-      </c>
-      <c r="E21" s="34">
-        <f>'BASE INOVAFARMA AGO.26'!I8</f>
-        <v/>
-      </c>
-      <c r="F21" s="34">
-        <f>'BASE INOVAFARMA AGO.26'!I9</f>
-        <v/>
-      </c>
-      <c r="G21" s="34">
-        <f>'BASE INOVAFARMA AGO.26'!I10</f>
-        <v/>
-      </c>
+          <t>1/3 CONSTITUCIONAL DE FÉRIAS</t>
+        </is>
+      </c>
+      <c r="B21" s="35" t="n"/>
+      <c r="C21" s="35" t="n"/>
+      <c r="D21" s="35" t="n"/>
+      <c r="E21" s="35" t="n"/>
+      <c r="F21" s="35" t="n"/>
+      <c r="G21" s="35" t="n"/>
       <c r="H21" s="20">
         <f>SUM(B21:G21)</f>
         <v/>
       </c>
       <c r="I21" s="33" t="inlineStr">
         <is>
-          <t>Populares, oficinais e similar normal.</t>
+          <t>Calculado pela contabilidade sobre o valor das férias.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="15" t="inlineStr">
-        <is>
-          <t>TOTAL DE PROVENTOS</t>
-        </is>
-      </c>
-      <c r="B22" s="20">
-        <f>SUM(B6:B21)-B9-B10</f>
-        <v/>
-      </c>
-      <c r="C22" s="20">
-        <f>SUM(C6:C21)-C9-C10</f>
-        <v/>
-      </c>
-      <c r="D22" s="20">
-        <f>SUM(D6:D21)-D9-D10</f>
-        <v/>
-      </c>
-      <c r="E22" s="20">
-        <f>SUM(E6:E21)-E9-E10</f>
-        <v/>
-      </c>
-      <c r="F22" s="20">
-        <f>SUM(F6:F21)-F9-F10</f>
-        <v/>
-      </c>
-      <c r="G22" s="20">
-        <f>SUM(G6:G21)-G9-G10</f>
+      <c r="A22" s="30" t="inlineStr">
+        <is>
+          <t>INCENTIVO APLICAÇÕES</t>
+        </is>
+      </c>
+      <c r="B22" s="34">
+        <f>'BASE INOVAFARMA AGO.26'!G5</f>
+        <v/>
+      </c>
+      <c r="C22" s="34">
+        <f>'BASE INOVAFARMA AGO.26'!G6</f>
+        <v/>
+      </c>
+      <c r="D22" s="34">
+        <f>'BASE INOVAFARMA AGO.26'!G7</f>
+        <v/>
+      </c>
+      <c r="E22" s="34">
+        <f>'BASE INOVAFARMA AGO.26'!G8</f>
+        <v/>
+      </c>
+      <c r="F22" s="34">
+        <f>'BASE INOVAFARMA AGO.26'!G9</f>
+        <v/>
+      </c>
+      <c r="G22" s="34">
+        <f>'BASE INOVAFARMA AGO.26'!G10</f>
         <v/>
       </c>
       <c r="H22" s="20">
@@ -2506,163 +2486,217 @@
       </c>
       <c r="I22" s="33" t="inlineStr">
         <is>
-          <t>Soma das rubricas acima (a linha COMISSÃO TOTAL já engloba a comissão do InovaFarma e o complemento).</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="19" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>DESCONTOS  (lançar com sinal negativo)</t>
-        </is>
-      </c>
-      <c r="B23" s="29" t="n"/>
-      <c r="C23" s="29" t="n"/>
-      <c r="D23" s="29" t="n"/>
-      <c r="E23" s="29" t="n"/>
-      <c r="F23" s="29" t="n"/>
-      <c r="G23" s="29" t="n"/>
-      <c r="H23" s="29" t="n"/>
-      <c r="I23" s="29" t="n"/>
+          <t>Incentivo de injetáveis apurado no InovaFarma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="30" t="inlineStr">
+        <is>
+          <t>INCENTIVO VITAMINAS</t>
+        </is>
+      </c>
+      <c r="B23" s="34">
+        <f>'BASE INOVAFARMA AGO.26'!H5</f>
+        <v/>
+      </c>
+      <c r="C23" s="34">
+        <f>'BASE INOVAFARMA AGO.26'!H6</f>
+        <v/>
+      </c>
+      <c r="D23" s="34">
+        <f>'BASE INOVAFARMA AGO.26'!H7</f>
+        <v/>
+      </c>
+      <c r="E23" s="34">
+        <f>'BASE INOVAFARMA AGO.26'!H8</f>
+        <v/>
+      </c>
+      <c r="F23" s="34">
+        <f>'BASE INOVAFARMA AGO.26'!H9</f>
+        <v/>
+      </c>
+      <c r="G23" s="34">
+        <f>'BASE INOVAFARMA AGO.26'!H10</f>
+        <v/>
+      </c>
+      <c r="H23" s="20">
+        <f>SUM(B23:G23)</f>
+        <v/>
+      </c>
+      <c r="I23" s="33" t="inlineStr">
+        <is>
+          <t>Grupo APLICAÇÃO E VITAMINAS INCENTIVO no InovaFarma.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="30" t="inlineStr">
         <is>
-          <t>ADIANTAMENTO SALARIAL / VALES</t>
-        </is>
-      </c>
-      <c r="B24" s="35" t="n"/>
-      <c r="C24" s="35" t="n"/>
-      <c r="D24" s="35" t="n"/>
-      <c r="E24" s="35" t="n"/>
-      <c r="F24" s="35" t="n"/>
-      <c r="G24" s="35" t="n"/>
+          <t>OUTROS INCENTIVOS</t>
+        </is>
+      </c>
+      <c r="B24" s="34">
+        <f>'BASE INOVAFARMA AGO.26'!I5</f>
+        <v/>
+      </c>
+      <c r="C24" s="34">
+        <f>'BASE INOVAFARMA AGO.26'!I6</f>
+        <v/>
+      </c>
+      <c r="D24" s="34">
+        <f>'BASE INOVAFARMA AGO.26'!I7</f>
+        <v/>
+      </c>
+      <c r="E24" s="34">
+        <f>'BASE INOVAFARMA AGO.26'!I8</f>
+        <v/>
+      </c>
+      <c r="F24" s="34">
+        <f>'BASE INOVAFARMA AGO.26'!I9</f>
+        <v/>
+      </c>
+      <c r="G24" s="34">
+        <f>'BASE INOVAFARMA AGO.26'!I10</f>
+        <v/>
+      </c>
       <c r="H24" s="20">
         <f>SUM(B24:G24)</f>
         <v/>
       </c>
       <c r="I24" s="33" t="inlineStr">
         <is>
-          <t>PREENCHER com os vales adiantados durante agosto.</t>
+          <t>Populares, oficinais e similar normal.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="30" t="inlineStr">
-        <is>
-          <t>ADIANT. VALES INCENT. E APLIC.</t>
-        </is>
-      </c>
-      <c r="B25" s="37">
-        <f>-(B19+B20+B21)</f>
-        <v/>
-      </c>
-      <c r="C25" s="37">
-        <f>-(C19+C20+C21)</f>
-        <v/>
-      </c>
-      <c r="D25" s="37">
-        <f>-(D19+D20+D21)</f>
-        <v/>
-      </c>
-      <c r="E25" s="37">
-        <f>-(E19+E20+E21)</f>
-        <v/>
-      </c>
-      <c r="F25" s="37">
-        <f>-(F19+F20+F21)</f>
-        <v/>
-      </c>
-      <c r="G25" s="37">
-        <f>-(G19+G20+G21)</f>
-        <v/>
-      </c>
-      <c r="H25" s="32">
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>TOTAL DE PROVENTOS</t>
+        </is>
+      </c>
+      <c r="B25" s="20">
+        <f>SUM(B6:B24)-B9-B10</f>
+        <v/>
+      </c>
+      <c r="C25" s="20">
+        <f>SUM(C6:C24)-C9-C10</f>
+        <v/>
+      </c>
+      <c r="D25" s="20">
+        <f>SUM(D6:D24)-D9-D10</f>
+        <v/>
+      </c>
+      <c r="E25" s="20">
+        <f>SUM(E6:E24)-E9-E10</f>
+        <v/>
+      </c>
+      <c r="F25" s="20">
+        <f>SUM(F6:F24)-F9-F10</f>
+        <v/>
+      </c>
+      <c r="G25" s="20">
+        <f>SUM(G6:G24)-G9-G10</f>
+        <v/>
+      </c>
+      <c r="H25" s="20">
         <f>SUM(B25:G25)</f>
         <v/>
       </c>
       <c r="I25" s="33" t="inlineStr">
         <is>
-          <t>Estorno dos incentivos já adiantados em dinheiro no mês. AJUSTAR se algum incentivo não foi adiantado.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="30" t="inlineStr">
-        <is>
-          <t>CONVÊNIO</t>
-        </is>
-      </c>
-      <c r="B26" s="35" t="n"/>
-      <c r="C26" s="35" t="n"/>
-      <c r="D26" s="35" t="n"/>
-      <c r="E26" s="35" t="n"/>
-      <c r="F26" s="35" t="n"/>
-      <c r="G26" s="35" t="n"/>
-      <c r="H26" s="20">
-        <f>SUM(B26:G26)</f>
-        <v/>
-      </c>
-      <c r="I26" s="33" t="inlineStr">
-        <is>
-          <t>PREENCHER conforme o convênio de agosto.</t>
-        </is>
-      </c>
+          <t>Soma das rubricas acima (a linha COMISSÃO TOTAL já engloba a comissão do InovaFarma e o complemento).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="19" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>DESCONTOS  (lançar com sinal negativo)</t>
+        </is>
+      </c>
+      <c r="B26" s="29" t="n"/>
+      <c r="C26" s="29" t="n"/>
+      <c r="D26" s="29" t="n"/>
+      <c r="E26" s="29" t="n"/>
+      <c r="F26" s="29" t="n"/>
+      <c r="G26" s="29" t="n"/>
+      <c r="H26" s="29" t="n"/>
+      <c r="I26" s="29" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="30" t="inlineStr">
         <is>
-          <t>DESCONTO FALTAS / ATRASOS</t>
-        </is>
-      </c>
-      <c r="B27" s="35" t="n"/>
-      <c r="C27" s="35" t="n"/>
-      <c r="D27" s="35" t="n"/>
-      <c r="E27" s="35" t="n"/>
-      <c r="F27" s="35" t="n"/>
-      <c r="G27" s="35" t="n"/>
-      <c r="H27" s="20">
+          <t>ADIANTAMENTO SALARIAL / VALES</t>
+        </is>
+      </c>
+      <c r="B27" s="31" t="n"/>
+      <c r="C27" s="31" t="n">
+        <v>-2192</v>
+      </c>
+      <c r="D27" s="31" t="n"/>
+      <c r="E27" s="31" t="n">
+        <v>-1955</v>
+      </c>
+      <c r="F27" s="31" t="n">
+        <v>-200</v>
+      </c>
+      <c r="G27" s="31" t="n"/>
+      <c r="H27" s="32">
         <f>SUM(B27:G27)</f>
         <v/>
       </c>
       <c r="I27" s="33" t="inlineStr">
         <is>
-          <t>PREENCHER conforme o ponto.</t>
+          <t>Rubrica 630 (Desconto - verbas / Adiantamento) do holerite da Betel.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="30" t="inlineStr">
         <is>
-          <t>DESCONTO VALE TRANSPORTE 6%</t>
-        </is>
-      </c>
-      <c r="B28" s="31" t="n"/>
-      <c r="C28" s="31" t="n">
-        <v>-84.29000000000001</v>
-      </c>
-      <c r="D28" s="31" t="n"/>
-      <c r="E28" s="31" t="n">
-        <v>-74.29000000000001</v>
-      </c>
-      <c r="F28" s="31" t="n">
-        <v>-84.29000000000001</v>
-      </c>
-      <c r="G28" s="31" t="n"/>
+          <t>ADIANT. VALES INCENT. E APLIC.</t>
+        </is>
+      </c>
+      <c r="B28" s="39">
+        <f>-(B22+B23+B24)</f>
+        <v/>
+      </c>
+      <c r="C28" s="39">
+        <f>-(C22+C23+C24)</f>
+        <v/>
+      </c>
+      <c r="D28" s="39">
+        <f>-(D22+D23+D24)</f>
+        <v/>
+      </c>
+      <c r="E28" s="39">
+        <f>-(E22+E23+E24)</f>
+        <v/>
+      </c>
+      <c r="F28" s="39">
+        <f>-(F22+F23+F24)</f>
+        <v/>
+      </c>
+      <c r="G28" s="39">
+        <f>-(G22+G23+G24)</f>
+        <v/>
+      </c>
       <c r="H28" s="32">
         <f>SUM(B28:G28)</f>
         <v/>
       </c>
       <c r="I28" s="33" t="inlineStr">
         <is>
-          <t>Valores praticados em jul/26. 6% sobre R$ 1.621,00 seria R$ 97,26 — CONFERIR a base usada. Quem passou o mês em férias fica sem desconto.</t>
+          <t>Estorno dos incentivos já adiantados em dinheiro no mês. AJUSTAR se algum incentivo não foi adiantado.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="30" t="inlineStr">
         <is>
-          <t>DESCONTO INSS</t>
+          <t>CONVÊNIO</t>
         </is>
       </c>
       <c r="B29" s="35" t="n"/>
@@ -2677,14 +2711,14 @@
       </c>
       <c r="I29" s="33" t="inlineStr">
         <is>
-          <t>A CALCULAR PELA CONTABILIDADE sobre o total de proventos.</t>
+          <t>PREENCHER conforme o convênio de agosto.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="30" t="inlineStr">
         <is>
-          <t>DESCONTO IRRF</t>
+          <t>DESCONTO FALTAS / ATRASOS</t>
         </is>
       </c>
       <c r="B30" s="35" t="n"/>
@@ -2699,171 +2733,206 @@
       </c>
       <c r="I30" s="33" t="inlineStr">
         <is>
-          <t>A CALCULAR PELA CONTABILIDADE.</t>
+          <t>PREENCHER conforme o ponto.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="15" t="inlineStr">
+      <c r="A31" s="30" t="inlineStr">
+        <is>
+          <t>DESCONTO VALE TRANSPORTE 6%</t>
+        </is>
+      </c>
+      <c r="B31" s="31" t="n"/>
+      <c r="C31" s="31" t="n">
+        <v>-84.29000000000001</v>
+      </c>
+      <c r="D31" s="31" t="n">
+        <v>-3.24</v>
+      </c>
+      <c r="E31" s="31" t="n">
+        <v>-68.08</v>
+      </c>
+      <c r="F31" s="31" t="n">
+        <v>-84.29000000000001</v>
+      </c>
+      <c r="G31" s="31" t="n"/>
+      <c r="H31" s="32">
+        <f>SUM(B31:G31)</f>
+        <v/>
+      </c>
+      <c r="I31" s="33" t="inlineStr">
+        <is>
+          <t>Rubrica 604 do holerite da Betel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="30" t="inlineStr">
+        <is>
+          <t>DESCONTO INSS</t>
+        </is>
+      </c>
+      <c r="B32" s="31" t="n">
+        <v>-592.27</v>
+      </c>
+      <c r="C32" s="31" t="n">
+        <v>-371.35</v>
+      </c>
+      <c r="D32" s="31" t="n"/>
+      <c r="E32" s="31" t="n">
+        <v>-235.06</v>
+      </c>
+      <c r="F32" s="31" t="n">
+        <v>-136.72</v>
+      </c>
+      <c r="G32" s="31" t="n"/>
+      <c r="H32" s="32">
+        <f>SUM(B32:G32)</f>
+        <v/>
+      </c>
+      <c r="I32" s="33" t="inlineStr">
+        <is>
+          <t>Rubrica 903 do holerite da Betel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="30" t="inlineStr">
+        <is>
+          <t>DESCONTO IRRF</t>
+        </is>
+      </c>
+      <c r="B33" s="31" t="n">
+        <v>-251.04</v>
+      </c>
+      <c r="C33" s="31" t="n"/>
+      <c r="D33" s="31" t="n"/>
+      <c r="E33" s="31" t="n"/>
+      <c r="F33" s="31" t="n"/>
+      <c r="G33" s="31" t="n"/>
+      <c r="H33" s="32">
+        <f>SUM(B33:G33)</f>
+        <v/>
+      </c>
+      <c r="I33" s="33" t="inlineStr">
+        <is>
+          <t>Rubrica 914 do holerite da Betel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="15" t="inlineStr">
         <is>
           <t>TOTAL DE DESCONTOS</t>
         </is>
       </c>
-      <c r="B31" s="20">
-        <f>SUM(B24:B30)</f>
-        <v/>
-      </c>
-      <c r="C31" s="20">
-        <f>SUM(C24:C30)</f>
-        <v/>
-      </c>
-      <c r="D31" s="20">
-        <f>SUM(D24:D30)</f>
-        <v/>
-      </c>
-      <c r="E31" s="20">
-        <f>SUM(E24:E30)</f>
-        <v/>
-      </c>
-      <c r="F31" s="20">
-        <f>SUM(F24:F30)</f>
-        <v/>
-      </c>
-      <c r="G31" s="20">
-        <f>SUM(G24:G30)</f>
-        <v/>
-      </c>
-      <c r="H31" s="20">
-        <f>SUM(B31:G31)</f>
-        <v/>
-      </c>
-      <c r="I31" s="33" t="inlineStr"/>
-    </row>
-    <row r="32" ht="19" customHeight="1">
-      <c r="A32" s="3" t="inlineStr">
+      <c r="B34" s="20">
+        <f>SUM(B27:B33)</f>
+        <v/>
+      </c>
+      <c r="C34" s="20">
+        <f>SUM(C27:C33)</f>
+        <v/>
+      </c>
+      <c r="D34" s="20">
+        <f>SUM(D27:D33)</f>
+        <v/>
+      </c>
+      <c r="E34" s="20">
+        <f>SUM(E27:E33)</f>
+        <v/>
+      </c>
+      <c r="F34" s="20">
+        <f>SUM(F27:F33)</f>
+        <v/>
+      </c>
+      <c r="G34" s="20">
+        <f>SUM(G27:G33)</f>
+        <v/>
+      </c>
+      <c r="H34" s="20">
+        <f>SUM(B34:G34)</f>
+        <v/>
+      </c>
+      <c r="I34" s="33" t="inlineStr"/>
+    </row>
+    <row r="35" ht="19" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>LÍQUIDO</t>
         </is>
       </c>
-      <c r="B32" s="29" t="n"/>
-      <c r="C32" s="29" t="n"/>
-      <c r="D32" s="29" t="n"/>
-      <c r="E32" s="29" t="n"/>
-      <c r="F32" s="29" t="n"/>
-      <c r="G32" s="29" t="n"/>
-      <c r="H32" s="29" t="n"/>
-      <c r="I32" s="29" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="15" t="inlineStr">
+      <c r="B35" s="29" t="n"/>
+      <c r="C35" s="29" t="n"/>
+      <c r="D35" s="29" t="n"/>
+      <c r="E35" s="29" t="n"/>
+      <c r="F35" s="29" t="n"/>
+      <c r="G35" s="29" t="n"/>
+      <c r="H35" s="29" t="n"/>
+      <c r="I35" s="29" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="15" t="inlineStr">
         <is>
           <t>LÍQUIDO A RECEBER (05/09/2026)</t>
         </is>
       </c>
-      <c r="B33" s="38">
-        <f>B22+B31</f>
-        <v/>
-      </c>
-      <c r="C33" s="38">
-        <f>C22+C31</f>
-        <v/>
-      </c>
-      <c r="D33" s="38">
-        <f>D22+D31</f>
-        <v/>
-      </c>
-      <c r="E33" s="38">
-        <f>E22+E31</f>
-        <v/>
-      </c>
-      <c r="F33" s="38">
-        <f>F22+F31</f>
-        <v/>
-      </c>
-      <c r="G33" s="38">
-        <f>G22+G31</f>
-        <v/>
-      </c>
-      <c r="H33" s="38">
-        <f>SUM(B33:G33)</f>
-        <v/>
-      </c>
-      <c r="I33" s="33" t="inlineStr">
+      <c r="B36" s="40">
+        <f>B25+B34</f>
+        <v/>
+      </c>
+      <c r="C36" s="40">
+        <f>C25+C34</f>
+        <v/>
+      </c>
+      <c r="D36" s="40">
+        <f>D25+D34</f>
+        <v/>
+      </c>
+      <c r="E36" s="40">
+        <f>E25+E34</f>
+        <v/>
+      </c>
+      <c r="F36" s="40">
+        <f>F25+F34</f>
+        <v/>
+      </c>
+      <c r="G36" s="40">
+        <f>G25+G34</f>
+        <v/>
+      </c>
+      <c r="H36" s="40">
+        <f>SUM(B36:G36)</f>
+        <v/>
+      </c>
+      <c r="I36" s="33" t="inlineStr">
         <is>
           <t>Total de proventos menos descontos. Só fica definitivo depois do INSS/IRRF da contabilidade.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="19" customHeight="1">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t>INFORMATIVO — PAGO PELA EMPRESA, NÃO ENTRA NO HOLERITE</t>
-        </is>
-      </c>
-      <c r="B34" s="29" t="n"/>
-      <c r="C34" s="29" t="n"/>
-      <c r="D34" s="29" t="n"/>
-      <c r="E34" s="29" t="n"/>
-      <c r="F34" s="29" t="n"/>
-      <c r="G34" s="29" t="n"/>
-      <c r="H34" s="29" t="n"/>
-      <c r="I34" s="29" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="30" t="inlineStr">
-        <is>
-          <t>VALE TRANSPORTE (compra set/26)</t>
-        </is>
-      </c>
-      <c r="B35" s="35" t="n"/>
-      <c r="C35" s="35" t="n"/>
-      <c r="D35" s="35" t="n"/>
-      <c r="E35" s="35" t="n"/>
-      <c r="F35" s="35" t="n"/>
-      <c r="G35" s="35" t="n"/>
-      <c r="H35" s="20">
-        <f>SUM(B35:G35)</f>
-        <v/>
-      </c>
-      <c r="I35" s="33" t="inlineStr">
-        <is>
-          <t>PREENCHER com as passagens compradas para setembro/2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="30" t="inlineStr">
-        <is>
-          <t>VALE ALIMENTAÇÃO FERIADOS E DOMINGOS</t>
-        </is>
-      </c>
-      <c r="B36" s="35" t="n"/>
-      <c r="C36" s="35" t="n"/>
-      <c r="D36" s="35" t="n"/>
-      <c r="E36" s="35" t="n"/>
-      <c r="F36" s="35" t="n"/>
-      <c r="G36" s="35" t="n"/>
-      <c r="H36" s="20">
-        <f>SUM(B36:G36)</f>
-        <v/>
-      </c>
-      <c r="I36" s="33" t="inlineStr">
-        <is>
-          <t>PREENCHER conforme escala de domingos e feriados.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="30" t="inlineStr">
         <is>
-          <t>FÉRIAS PAGAS À PARTE (CONTAS A PAGAR)</t>
-        </is>
-      </c>
-      <c r="B37" s="31" t="n"/>
-      <c r="C37" s="31" t="n"/>
-      <c r="D37" s="31" t="n"/>
-      <c r="E37" s="31" t="n"/>
-      <c r="F37" s="31" t="n"/>
+          <t>LÍQUIDO DO HOLERITE (BETEL)</t>
+        </is>
+      </c>
+      <c r="B37" s="31" t="n">
+        <v>4805.1</v>
+      </c>
+      <c r="C37" s="31" t="n">
+        <v>1375.37</v>
+      </c>
+      <c r="D37" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="31" t="n">
+        <v>623.87</v>
+      </c>
+      <c r="F37" s="31" t="n">
+        <v>1368.35</v>
+      </c>
       <c r="G37" s="31" t="n"/>
       <c r="H37" s="32">
         <f>SUM(B37:G37)</f>
@@ -2871,76 +2940,197 @@
       </c>
       <c r="I37" s="33" t="inlineStr">
         <is>
+          <t>Valor líquido do demonstrativo emitido pela Betel Contabilidade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="15" t="inlineStr">
+        <is>
+          <t>DIFERENÇA (planilha − holerite)</t>
+        </is>
+      </c>
+      <c r="B38" s="20">
+        <f>ROUND(B36-B37,2)</f>
+        <v/>
+      </c>
+      <c r="C38" s="20">
+        <f>ROUND(C36-C37,2)</f>
+        <v/>
+      </c>
+      <c r="D38" s="20">
+        <f>ROUND(D36-D37,2)</f>
+        <v/>
+      </c>
+      <c r="E38" s="20">
+        <f>ROUND(E36-E37,2)</f>
+        <v/>
+      </c>
+      <c r="F38" s="20">
+        <f>ROUND(F36-F37,2)</f>
+        <v/>
+      </c>
+      <c r="G38" s="20">
+        <f>ROUND(G36-G37,2)</f>
+        <v/>
+      </c>
+      <c r="H38" s="20">
+        <f>SUM(B38:G38)</f>
+        <v/>
+      </c>
+      <c r="I38" s="33" t="inlineStr">
+        <is>
+          <t>Deve ser zero. Os incentivos entram como provento e como desconto, então não afetam o líquido.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="19" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>INFORMATIVO — PAGO PELA EMPRESA, NÃO ENTRA NO HOLERITE</t>
+        </is>
+      </c>
+      <c r="B39" s="29" t="n"/>
+      <c r="C39" s="29" t="n"/>
+      <c r="D39" s="29" t="n"/>
+      <c r="E39" s="29" t="n"/>
+      <c r="F39" s="29" t="n"/>
+      <c r="G39" s="29" t="n"/>
+      <c r="H39" s="29" t="n"/>
+      <c r="I39" s="29" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="30" t="inlineStr">
+        <is>
+          <t>VALE TRANSPORTE (compra set/26)</t>
+        </is>
+      </c>
+      <c r="B40" s="35" t="n"/>
+      <c r="C40" s="35" t="n"/>
+      <c r="D40" s="35" t="n"/>
+      <c r="E40" s="35" t="n"/>
+      <c r="F40" s="35" t="n"/>
+      <c r="G40" s="35" t="n"/>
+      <c r="H40" s="20">
+        <f>SUM(B40:G40)</f>
+        <v/>
+      </c>
+      <c r="I40" s="33" t="inlineStr">
+        <is>
+          <t>PREENCHER com as passagens compradas para setembro/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="30" t="inlineStr">
+        <is>
+          <t>VALE ALIMENTAÇÃO FERIADOS E DOMINGOS</t>
+        </is>
+      </c>
+      <c r="B41" s="35" t="n"/>
+      <c r="C41" s="35" t="n"/>
+      <c r="D41" s="35" t="n"/>
+      <c r="E41" s="35" t="n"/>
+      <c r="F41" s="35" t="n"/>
+      <c r="G41" s="35" t="n"/>
+      <c r="H41" s="20">
+        <f>SUM(B41:G41)</f>
+        <v/>
+      </c>
+      <c r="I41" s="33" t="inlineStr">
+        <is>
+          <t>PREENCHER conforme escala de domingos e feriados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="30" t="inlineStr">
+        <is>
+          <t>FÉRIAS PAGAS À PARTE (CONTAS A PAGAR)</t>
+        </is>
+      </c>
+      <c r="B42" s="31" t="n"/>
+      <c r="C42" s="31" t="n"/>
+      <c r="D42" s="31" t="n"/>
+      <c r="E42" s="31" t="n"/>
+      <c r="F42" s="31" t="n"/>
+      <c r="G42" s="31" t="n"/>
+      <c r="H42" s="32">
+        <f>SUM(B42:G42)</f>
+        <v/>
+      </c>
+      <c r="I42" s="33" t="inlineStr">
+        <is>
           <t>Recibo de férias pago fora do holerite — lembrete para o contas a pagar. GENECIR: férias de 01 a 30/08/2026, pagas em recibo próprio — informar o valor.</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="21" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="21" t="inlineStr">
         <is>
           <t>LEGENDA</t>
         </is>
       </c>
-      <c r="B39" s="22" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="21" t="inlineStr">
+      <c r="B44" s="22" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="21" t="inlineStr">
         <is>
           <t>Célula amarela, texto azul</t>
         </is>
       </c>
-      <c r="B40" s="22" t="inlineStr">
+      <c r="B45" s="22" t="inlineStr">
         <is>
           <t>valor digitado — PREENCHER ou conferir antes de enviar.</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="21" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="21" t="inlineStr">
         <is>
           <t>Célula laranja</t>
         </is>
       </c>
-      <c r="B41" s="22" t="inlineStr">
+      <c r="B46" s="22" t="inlineStr">
         <is>
           <t>valor repetido de julho/2026 — CONFERIR se continua válido em agosto.</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="21" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="21" t="inlineStr">
         <is>
           <t>Texto verde</t>
         </is>
       </c>
-      <c r="B42" s="22" t="inlineStr">
+      <c r="B47" s="22" t="inlineStr">
         <is>
           <t>valor puxado da aba BASE INOVAFARMA AGO.26 (não digitar por cima).</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="21" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="21" t="inlineStr">
         <is>
           <t>Texto preto em célula verde</t>
         </is>
       </c>
-      <c r="B43" s="22" t="inlineStr">
+      <c r="B48" s="22" t="inlineStr">
         <is>
           <t>resultado de fórmula — não alterar.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I37"/>
+  <autoFilter ref="A4:I42"/>
   <mergeCells count="7">
+    <mergeCell ref="B44:I44"/>
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="B39:I39"/>
+    <mergeCell ref="B48:I48"/>
+    <mergeCell ref="B47:I47"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="B42:I42"/>
-    <mergeCell ref="B43:I43"/>
-    <mergeCell ref="B41:I41"/>
-    <mergeCell ref="B40:I40"/>
+    <mergeCell ref="B45:I45"/>
+    <mergeCell ref="B46:I46"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3518,31 +3708,31 @@
           <t>LÍQUIDO PAGO (05/08/2026)</t>
         </is>
       </c>
-      <c r="B26" s="38">
+      <c r="B26" s="40">
         <f>B16+B24</f>
         <v/>
       </c>
-      <c r="C26" s="38">
+      <c r="C26" s="40">
         <f>C16+C24</f>
         <v/>
       </c>
-      <c r="D26" s="38">
+      <c r="D26" s="40">
         <f>D16+D24</f>
         <v/>
       </c>
-      <c r="E26" s="38">
+      <c r="E26" s="40">
         <f>E16+E24</f>
         <v/>
       </c>
-      <c r="F26" s="38">
+      <c r="F26" s="40">
         <f>F16+F24</f>
         <v/>
       </c>
-      <c r="G26" s="38">
+      <c r="G26" s="40">
         <f>G16+G24</f>
         <v/>
       </c>
-      <c r="H26" s="38">
+      <c r="H26" s="40">
         <f>SUM(B26:G26)</f>
         <v/>
       </c>
@@ -3803,35 +3993,35 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="39" t="inlineStr">
+      <c r="A36" s="41" t="inlineStr">
         <is>
           <t>AJUSTES FEITOS NESTA REVISÃO (a planilha original continua intacta):</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="40" t="inlineStr">
+      <c r="A37" s="42" t="inlineStr">
         <is>
           <t>1. Rubricas separadas em PROVENTOS × DESCONTOS, com subtotais próprios.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="40" t="inlineStr">
+      <c r="A38" s="42" t="inlineStr">
         <is>
           <t>2. Nomes de rubrica padronizados e coluna de observação com a origem de cada valor.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="40" t="inlineStr">
+      <c r="A39" s="42" t="inlineStr">
         <is>
           <t>3. Conferência do DSR: em julho foi usado o fator de agosto (5/26) em vez de 4/27.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="40" t="inlineStr">
+      <c r="A40" s="42" t="inlineStr">
         <is>
           <t>4. Linha de conferência comparando o líquido revisado com o SALDO FINAL da planilha original (tem que fechar em zero).</t>
         </is>
@@ -3929,7 +4119,7 @@
         <f>'HOLERITE AGO.26'!B6</f>
         <v/>
       </c>
-      <c r="E5" s="41" t="n"/>
+      <c r="E5" s="43" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="30" t="inlineStr">
@@ -3951,7 +4141,7 @@
         <f>'HOLERITE AGO.26'!B7</f>
         <v/>
       </c>
-      <c r="E6" s="41" t="n"/>
+      <c r="E6" s="43" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="30" t="inlineStr">
@@ -3973,7 +4163,7 @@
         <f>'HOLERITE AGO.26'!B8</f>
         <v/>
       </c>
-      <c r="E7" s="41" t="n"/>
+      <c r="E7" s="43" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="30" t="inlineStr">
@@ -3995,7 +4185,7 @@
         <f>'HOLERITE AGO.26'!B11</f>
         <v/>
       </c>
-      <c r="E8" s="41" t="n"/>
+      <c r="E8" s="43" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="30" t="inlineStr">
@@ -4017,7 +4207,7 @@
         <f>'HOLERITE AGO.26'!B12</f>
         <v/>
       </c>
-      <c r="E9" s="41" t="n"/>
+      <c r="E9" s="43" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="30" t="inlineStr">
@@ -4036,10 +4226,10 @@
         </is>
       </c>
       <c r="D10" s="34">
-        <f>'HOLERITE AGO.26'!B13</f>
-        <v/>
-      </c>
-      <c r="E10" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!B16</f>
+        <v/>
+      </c>
+      <c r="E10" s="43" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="30" t="inlineStr">
@@ -4058,10 +4248,10 @@
         </is>
       </c>
       <c r="D11" s="34">
-        <f>'HOLERITE AGO.26'!B14</f>
-        <v/>
-      </c>
-      <c r="E11" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!B17</f>
+        <v/>
+      </c>
+      <c r="E11" s="43" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="30" t="inlineStr">
@@ -4080,10 +4270,10 @@
         </is>
       </c>
       <c r="D12" s="34">
-        <f>'HOLERITE AGO.26'!B15</f>
-        <v/>
-      </c>
-      <c r="E12" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!B18</f>
+        <v/>
+      </c>
+      <c r="E12" s="43" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="30" t="inlineStr">
@@ -4102,10 +4292,10 @@
         </is>
       </c>
       <c r="D13" s="34">
-        <f>'HOLERITE AGO.26'!B16</f>
-        <v/>
-      </c>
-      <c r="E13" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!B19</f>
+        <v/>
+      </c>
+      <c r="E13" s="43" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="30" t="inlineStr">
@@ -4124,10 +4314,10 @@
         </is>
       </c>
       <c r="D14" s="34">
-        <f>'HOLERITE AGO.26'!B17</f>
-        <v/>
-      </c>
-      <c r="E14" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!B20</f>
+        <v/>
+      </c>
+      <c r="E14" s="43" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="30" t="inlineStr">
@@ -4146,10 +4336,10 @@
         </is>
       </c>
       <c r="D15" s="34">
-        <f>'HOLERITE AGO.26'!B18</f>
-        <v/>
-      </c>
-      <c r="E15" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!B21</f>
+        <v/>
+      </c>
+      <c r="E15" s="43" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="30" t="inlineStr">
@@ -4168,10 +4358,10 @@
         </is>
       </c>
       <c r="D16" s="34">
-        <f>'HOLERITE AGO.26'!B19</f>
-        <v/>
-      </c>
-      <c r="E16" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!B22</f>
+        <v/>
+      </c>
+      <c r="E16" s="43" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="30" t="inlineStr">
@@ -4190,10 +4380,10 @@
         </is>
       </c>
       <c r="D17" s="34">
-        <f>'HOLERITE AGO.26'!B20</f>
-        <v/>
-      </c>
-      <c r="E17" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!B23</f>
+        <v/>
+      </c>
+      <c r="E17" s="43" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="30" t="inlineStr">
@@ -4212,29 +4402,29 @@
         </is>
       </c>
       <c r="D18" s="34">
-        <f>'HOLERITE AGO.26'!B21</f>
-        <v/>
-      </c>
-      <c r="E18" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!B24</f>
+        <v/>
+      </c>
+      <c r="E18" s="43" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="42" t="inlineStr">
+      <c r="A19" s="44" t="inlineStr">
         <is>
           <t>ARIANE</t>
         </is>
       </c>
-      <c r="B19" s="42" t="inlineStr">
+      <c r="B19" s="44" t="inlineStr">
         <is>
           <t>TOTAL DE PROVENTOS</t>
         </is>
       </c>
-      <c r="C19" s="42" t="inlineStr">
+      <c r="C19" s="44" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="D19" s="43">
-        <f>'HOLERITE AGO.26'!B22</f>
+      <c r="D19" s="45">
+        <f>'HOLERITE AGO.26'!B25</f>
         <v/>
       </c>
       <c r="E19" s="18" t="n"/>
@@ -4256,10 +4446,10 @@
         </is>
       </c>
       <c r="D20" s="34">
-        <f>'HOLERITE AGO.26'!B24</f>
-        <v/>
-      </c>
-      <c r="E20" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!B27</f>
+        <v/>
+      </c>
+      <c r="E20" s="43" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="30" t="inlineStr">
@@ -4278,10 +4468,10 @@
         </is>
       </c>
       <c r="D21" s="34">
-        <f>'HOLERITE AGO.26'!B25</f>
-        <v/>
-      </c>
-      <c r="E21" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!B28</f>
+        <v/>
+      </c>
+      <c r="E21" s="43" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="30" t="inlineStr">
@@ -4300,10 +4490,10 @@
         </is>
       </c>
       <c r="D22" s="34">
-        <f>'HOLERITE AGO.26'!B26</f>
-        <v/>
-      </c>
-      <c r="E22" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!B29</f>
+        <v/>
+      </c>
+      <c r="E22" s="43" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="30" t="inlineStr">
@@ -4322,10 +4512,10 @@
         </is>
       </c>
       <c r="D23" s="34">
-        <f>'HOLERITE AGO.26'!B27</f>
-        <v/>
-      </c>
-      <c r="E23" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!B30</f>
+        <v/>
+      </c>
+      <c r="E23" s="43" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="30" t="inlineStr">
@@ -4344,10 +4534,10 @@
         </is>
       </c>
       <c r="D24" s="34">
-        <f>'HOLERITE AGO.26'!B28</f>
-        <v/>
-      </c>
-      <c r="E24" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!B31</f>
+        <v/>
+      </c>
+      <c r="E24" s="43" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="30" t="inlineStr">
@@ -4366,10 +4556,10 @@
         </is>
       </c>
       <c r="D25" s="34">
-        <f>'HOLERITE AGO.26'!B29</f>
-        <v/>
-      </c>
-      <c r="E25" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!B32</f>
+        <v/>
+      </c>
+      <c r="E25" s="43" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="30" t="inlineStr">
@@ -4388,54 +4578,54 @@
         </is>
       </c>
       <c r="D26" s="34">
-        <f>'HOLERITE AGO.26'!B30</f>
-        <v/>
-      </c>
-      <c r="E26" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!B33</f>
+        <v/>
+      </c>
+      <c r="E26" s="43" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="42" t="inlineStr">
+      <c r="A27" s="44" t="inlineStr">
         <is>
           <t>ARIANE</t>
         </is>
       </c>
-      <c r="B27" s="42" t="inlineStr">
+      <c r="B27" s="44" t="inlineStr">
         <is>
           <t>TOTAL DE DESCONTOS</t>
         </is>
       </c>
-      <c r="C27" s="42" t="inlineStr">
+      <c r="C27" s="44" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="D27" s="43">
-        <f>'HOLERITE AGO.26'!B31</f>
+      <c r="D27" s="45">
+        <f>'HOLERITE AGO.26'!B34</f>
         <v/>
       </c>
       <c r="E27" s="18" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="44" t="inlineStr">
+      <c r="A28" s="46" t="inlineStr">
         <is>
           <t>ARIANE</t>
         </is>
       </c>
-      <c r="B28" s="45" t="inlineStr">
+      <c r="B28" s="47" t="inlineStr">
         <is>
           <t>LÍQUIDO A RECEBER</t>
         </is>
       </c>
-      <c r="C28" s="45" t="inlineStr">
+      <c r="C28" s="47" t="inlineStr">
         <is>
           <t>Líquido</t>
         </is>
       </c>
-      <c r="D28" s="46">
-        <f>'HOLERITE AGO.26'!B33</f>
-        <v/>
-      </c>
-      <c r="E28" s="47" t="n"/>
+      <c r="D28" s="48">
+        <f>'HOLERITE AGO.26'!B36</f>
+        <v/>
+      </c>
+      <c r="E28" s="49" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="30" t="inlineStr">
@@ -4457,7 +4647,7 @@
         <f>'HOLERITE AGO.26'!C6</f>
         <v/>
       </c>
-      <c r="E30" s="41" t="n"/>
+      <c r="E30" s="43" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="30" t="inlineStr">
@@ -4479,7 +4669,7 @@
         <f>'HOLERITE AGO.26'!C7</f>
         <v/>
       </c>
-      <c r="E31" s="41" t="n"/>
+      <c r="E31" s="43" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="30" t="inlineStr">
@@ -4501,7 +4691,7 @@
         <f>'HOLERITE AGO.26'!C8</f>
         <v/>
       </c>
-      <c r="E32" s="41" t="n"/>
+      <c r="E32" s="43" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="30" t="inlineStr">
@@ -4523,7 +4713,7 @@
         <f>'HOLERITE AGO.26'!C11</f>
         <v/>
       </c>
-      <c r="E33" s="41" t="n"/>
+      <c r="E33" s="43" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="30" t="inlineStr">
@@ -4545,7 +4735,7 @@
         <f>'HOLERITE AGO.26'!C12</f>
         <v/>
       </c>
-      <c r="E34" s="41" t="n"/>
+      <c r="E34" s="43" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="30" t="inlineStr">
@@ -4564,10 +4754,10 @@
         </is>
       </c>
       <c r="D35" s="34">
-        <f>'HOLERITE AGO.26'!C13</f>
-        <v/>
-      </c>
-      <c r="E35" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!C16</f>
+        <v/>
+      </c>
+      <c r="E35" s="43" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="30" t="inlineStr">
@@ -4586,10 +4776,10 @@
         </is>
       </c>
       <c r="D36" s="34">
-        <f>'HOLERITE AGO.26'!C14</f>
-        <v/>
-      </c>
-      <c r="E36" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!C17</f>
+        <v/>
+      </c>
+      <c r="E36" s="43" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="30" t="inlineStr">
@@ -4608,10 +4798,10 @@
         </is>
       </c>
       <c r="D37" s="34">
-        <f>'HOLERITE AGO.26'!C15</f>
-        <v/>
-      </c>
-      <c r="E37" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!C18</f>
+        <v/>
+      </c>
+      <c r="E37" s="43" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="30" t="inlineStr">
@@ -4630,10 +4820,10 @@
         </is>
       </c>
       <c r="D38" s="34">
-        <f>'HOLERITE AGO.26'!C16</f>
-        <v/>
-      </c>
-      <c r="E38" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!C19</f>
+        <v/>
+      </c>
+      <c r="E38" s="43" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="30" t="inlineStr">
@@ -4652,10 +4842,10 @@
         </is>
       </c>
       <c r="D39" s="34">
-        <f>'HOLERITE AGO.26'!C17</f>
-        <v/>
-      </c>
-      <c r="E39" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!C20</f>
+        <v/>
+      </c>
+      <c r="E39" s="43" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="30" t="inlineStr">
@@ -4674,10 +4864,10 @@
         </is>
       </c>
       <c r="D40" s="34">
-        <f>'HOLERITE AGO.26'!C18</f>
-        <v/>
-      </c>
-      <c r="E40" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!C21</f>
+        <v/>
+      </c>
+      <c r="E40" s="43" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="30" t="inlineStr">
@@ -4696,10 +4886,10 @@
         </is>
       </c>
       <c r="D41" s="34">
-        <f>'HOLERITE AGO.26'!C19</f>
-        <v/>
-      </c>
-      <c r="E41" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!C22</f>
+        <v/>
+      </c>
+      <c r="E41" s="43" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="30" t="inlineStr">
@@ -4718,10 +4908,10 @@
         </is>
       </c>
       <c r="D42" s="34">
-        <f>'HOLERITE AGO.26'!C20</f>
-        <v/>
-      </c>
-      <c r="E42" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!C23</f>
+        <v/>
+      </c>
+      <c r="E42" s="43" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="30" t="inlineStr">
@@ -4740,29 +4930,29 @@
         </is>
       </c>
       <c r="D43" s="34">
-        <f>'HOLERITE AGO.26'!C21</f>
-        <v/>
-      </c>
-      <c r="E43" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!C24</f>
+        <v/>
+      </c>
+      <c r="E43" s="43" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="42" t="inlineStr">
+      <c r="A44" s="44" t="inlineStr">
         <is>
           <t>ELIANA</t>
         </is>
       </c>
-      <c r="B44" s="42" t="inlineStr">
+      <c r="B44" s="44" t="inlineStr">
         <is>
           <t>TOTAL DE PROVENTOS</t>
         </is>
       </c>
-      <c r="C44" s="42" t="inlineStr">
+      <c r="C44" s="44" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="D44" s="43">
-        <f>'HOLERITE AGO.26'!C22</f>
+      <c r="D44" s="45">
+        <f>'HOLERITE AGO.26'!C25</f>
         <v/>
       </c>
       <c r="E44" s="18" t="n"/>
@@ -4784,10 +4974,10 @@
         </is>
       </c>
       <c r="D45" s="34">
-        <f>'HOLERITE AGO.26'!C24</f>
-        <v/>
-      </c>
-      <c r="E45" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!C27</f>
+        <v/>
+      </c>
+      <c r="E45" s="43" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="30" t="inlineStr">
@@ -4806,10 +4996,10 @@
         </is>
       </c>
       <c r="D46" s="34">
-        <f>'HOLERITE AGO.26'!C25</f>
-        <v/>
-      </c>
-      <c r="E46" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!C28</f>
+        <v/>
+      </c>
+      <c r="E46" s="43" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="30" t="inlineStr">
@@ -4828,10 +5018,10 @@
         </is>
       </c>
       <c r="D47" s="34">
-        <f>'HOLERITE AGO.26'!C26</f>
-        <v/>
-      </c>
-      <c r="E47" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!C29</f>
+        <v/>
+      </c>
+      <c r="E47" s="43" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="30" t="inlineStr">
@@ -4850,10 +5040,10 @@
         </is>
       </c>
       <c r="D48" s="34">
-        <f>'HOLERITE AGO.26'!C27</f>
-        <v/>
-      </c>
-      <c r="E48" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!C30</f>
+        <v/>
+      </c>
+      <c r="E48" s="43" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="30" t="inlineStr">
@@ -4872,10 +5062,10 @@
         </is>
       </c>
       <c r="D49" s="34">
-        <f>'HOLERITE AGO.26'!C28</f>
-        <v/>
-      </c>
-      <c r="E49" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!C31</f>
+        <v/>
+      </c>
+      <c r="E49" s="43" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="30" t="inlineStr">
@@ -4894,10 +5084,10 @@
         </is>
       </c>
       <c r="D50" s="34">
-        <f>'HOLERITE AGO.26'!C29</f>
-        <v/>
-      </c>
-      <c r="E50" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!C32</f>
+        <v/>
+      </c>
+      <c r="E50" s="43" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="30" t="inlineStr">
@@ -4916,54 +5106,54 @@
         </is>
       </c>
       <c r="D51" s="34">
-        <f>'HOLERITE AGO.26'!C30</f>
-        <v/>
-      </c>
-      <c r="E51" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!C33</f>
+        <v/>
+      </c>
+      <c r="E51" s="43" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="42" t="inlineStr">
+      <c r="A52" s="44" t="inlineStr">
         <is>
           <t>ELIANA</t>
         </is>
       </c>
-      <c r="B52" s="42" t="inlineStr">
+      <c r="B52" s="44" t="inlineStr">
         <is>
           <t>TOTAL DE DESCONTOS</t>
         </is>
       </c>
-      <c r="C52" s="42" t="inlineStr">
+      <c r="C52" s="44" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="D52" s="43">
-        <f>'HOLERITE AGO.26'!C31</f>
+      <c r="D52" s="45">
+        <f>'HOLERITE AGO.26'!C34</f>
         <v/>
       </c>
       <c r="E52" s="18" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="44" t="inlineStr">
+      <c r="A53" s="46" t="inlineStr">
         <is>
           <t>ELIANA</t>
         </is>
       </c>
-      <c r="B53" s="45" t="inlineStr">
+      <c r="B53" s="47" t="inlineStr">
         <is>
           <t>LÍQUIDO A RECEBER</t>
         </is>
       </c>
-      <c r="C53" s="45" t="inlineStr">
+      <c r="C53" s="47" t="inlineStr">
         <is>
           <t>Líquido</t>
         </is>
       </c>
-      <c r="D53" s="46">
-        <f>'HOLERITE AGO.26'!C33</f>
-        <v/>
-      </c>
-      <c r="E53" s="47" t="n"/>
+      <c r="D53" s="48">
+        <f>'HOLERITE AGO.26'!C36</f>
+        <v/>
+      </c>
+      <c r="E53" s="49" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="30" t="inlineStr">
@@ -4985,7 +5175,7 @@
         <f>'HOLERITE AGO.26'!D6</f>
         <v/>
       </c>
-      <c r="E55" s="41" t="n"/>
+      <c r="E55" s="43" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="30" t="inlineStr">
@@ -5007,7 +5197,7 @@
         <f>'HOLERITE AGO.26'!D7</f>
         <v/>
       </c>
-      <c r="E56" s="41" t="n"/>
+      <c r="E56" s="43" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="30" t="inlineStr">
@@ -5029,7 +5219,7 @@
         <f>'HOLERITE AGO.26'!D8</f>
         <v/>
       </c>
-      <c r="E57" s="41" t="n"/>
+      <c r="E57" s="43" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="30" t="inlineStr">
@@ -5051,7 +5241,7 @@
         <f>'HOLERITE AGO.26'!D11</f>
         <v/>
       </c>
-      <c r="E58" s="41" t="n"/>
+      <c r="E58" s="43" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="30" t="inlineStr">
@@ -5073,7 +5263,7 @@
         <f>'HOLERITE AGO.26'!D12</f>
         <v/>
       </c>
-      <c r="E59" s="41" t="n"/>
+      <c r="E59" s="43" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="30" t="inlineStr">
@@ -5092,10 +5282,10 @@
         </is>
       </c>
       <c r="D60" s="34">
-        <f>'HOLERITE AGO.26'!D13</f>
-        <v/>
-      </c>
-      <c r="E60" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!D16</f>
+        <v/>
+      </c>
+      <c r="E60" s="43" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="30" t="inlineStr">
@@ -5114,10 +5304,10 @@
         </is>
       </c>
       <c r="D61" s="34">
-        <f>'HOLERITE AGO.26'!D14</f>
-        <v/>
-      </c>
-      <c r="E61" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!D17</f>
+        <v/>
+      </c>
+      <c r="E61" s="43" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="30" t="inlineStr">
@@ -5136,10 +5326,10 @@
         </is>
       </c>
       <c r="D62" s="34">
-        <f>'HOLERITE AGO.26'!D15</f>
-        <v/>
-      </c>
-      <c r="E62" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!D18</f>
+        <v/>
+      </c>
+      <c r="E62" s="43" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="30" t="inlineStr">
@@ -5158,10 +5348,10 @@
         </is>
       </c>
       <c r="D63" s="34">
-        <f>'HOLERITE AGO.26'!D16</f>
-        <v/>
-      </c>
-      <c r="E63" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!D19</f>
+        <v/>
+      </c>
+      <c r="E63" s="43" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="30" t="inlineStr">
@@ -5180,10 +5370,10 @@
         </is>
       </c>
       <c r="D64" s="34">
-        <f>'HOLERITE AGO.26'!D17</f>
-        <v/>
-      </c>
-      <c r="E64" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!D20</f>
+        <v/>
+      </c>
+      <c r="E64" s="43" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="30" t="inlineStr">
@@ -5202,10 +5392,10 @@
         </is>
       </c>
       <c r="D65" s="34">
-        <f>'HOLERITE AGO.26'!D18</f>
-        <v/>
-      </c>
-      <c r="E65" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!D21</f>
+        <v/>
+      </c>
+      <c r="E65" s="43" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="30" t="inlineStr">
@@ -5224,10 +5414,10 @@
         </is>
       </c>
       <c r="D66" s="34">
-        <f>'HOLERITE AGO.26'!D19</f>
-        <v/>
-      </c>
-      <c r="E66" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!D22</f>
+        <v/>
+      </c>
+      <c r="E66" s="43" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="30" t="inlineStr">
@@ -5246,10 +5436,10 @@
         </is>
       </c>
       <c r="D67" s="34">
-        <f>'HOLERITE AGO.26'!D20</f>
-        <v/>
-      </c>
-      <c r="E67" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!D23</f>
+        <v/>
+      </c>
+      <c r="E67" s="43" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="30" t="inlineStr">
@@ -5268,29 +5458,29 @@
         </is>
       </c>
       <c r="D68" s="34">
-        <f>'HOLERITE AGO.26'!D21</f>
-        <v/>
-      </c>
-      <c r="E68" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!D24</f>
+        <v/>
+      </c>
+      <c r="E68" s="43" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="42" t="inlineStr">
+      <c r="A69" s="44" t="inlineStr">
         <is>
           <t>GENECIR</t>
         </is>
       </c>
-      <c r="B69" s="42" t="inlineStr">
+      <c r="B69" s="44" t="inlineStr">
         <is>
           <t>TOTAL DE PROVENTOS</t>
         </is>
       </c>
-      <c r="C69" s="42" t="inlineStr">
+      <c r="C69" s="44" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="D69" s="43">
-        <f>'HOLERITE AGO.26'!D22</f>
+      <c r="D69" s="45">
+        <f>'HOLERITE AGO.26'!D25</f>
         <v/>
       </c>
       <c r="E69" s="18" t="n"/>
@@ -5312,10 +5502,10 @@
         </is>
       </c>
       <c r="D70" s="34">
-        <f>'HOLERITE AGO.26'!D24</f>
-        <v/>
-      </c>
-      <c r="E70" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!D27</f>
+        <v/>
+      </c>
+      <c r="E70" s="43" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="30" t="inlineStr">
@@ -5334,10 +5524,10 @@
         </is>
       </c>
       <c r="D71" s="34">
-        <f>'HOLERITE AGO.26'!D25</f>
-        <v/>
-      </c>
-      <c r="E71" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!D28</f>
+        <v/>
+      </c>
+      <c r="E71" s="43" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="30" t="inlineStr">
@@ -5356,10 +5546,10 @@
         </is>
       </c>
       <c r="D72" s="34">
-        <f>'HOLERITE AGO.26'!D26</f>
-        <v/>
-      </c>
-      <c r="E72" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!D29</f>
+        <v/>
+      </c>
+      <c r="E72" s="43" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="30" t="inlineStr">
@@ -5378,10 +5568,10 @@
         </is>
       </c>
       <c r="D73" s="34">
-        <f>'HOLERITE AGO.26'!D27</f>
-        <v/>
-      </c>
-      <c r="E73" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!D30</f>
+        <v/>
+      </c>
+      <c r="E73" s="43" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="30" t="inlineStr">
@@ -5400,10 +5590,10 @@
         </is>
       </c>
       <c r="D74" s="34">
-        <f>'HOLERITE AGO.26'!D28</f>
-        <v/>
-      </c>
-      <c r="E74" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!D31</f>
+        <v/>
+      </c>
+      <c r="E74" s="43" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="30" t="inlineStr">
@@ -5422,10 +5612,10 @@
         </is>
       </c>
       <c r="D75" s="34">
-        <f>'HOLERITE AGO.26'!D29</f>
-        <v/>
-      </c>
-      <c r="E75" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!D32</f>
+        <v/>
+      </c>
+      <c r="E75" s="43" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="30" t="inlineStr">
@@ -5444,54 +5634,54 @@
         </is>
       </c>
       <c r="D76" s="34">
-        <f>'HOLERITE AGO.26'!D30</f>
-        <v/>
-      </c>
-      <c r="E76" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!D33</f>
+        <v/>
+      </c>
+      <c r="E76" s="43" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="42" t="inlineStr">
+      <c r="A77" s="44" t="inlineStr">
         <is>
           <t>GENECIR</t>
         </is>
       </c>
-      <c r="B77" s="42" t="inlineStr">
+      <c r="B77" s="44" t="inlineStr">
         <is>
           <t>TOTAL DE DESCONTOS</t>
         </is>
       </c>
-      <c r="C77" s="42" t="inlineStr">
+      <c r="C77" s="44" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="D77" s="43">
-        <f>'HOLERITE AGO.26'!D31</f>
+      <c r="D77" s="45">
+        <f>'HOLERITE AGO.26'!D34</f>
         <v/>
       </c>
       <c r="E77" s="18" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="44" t="inlineStr">
+      <c r="A78" s="46" t="inlineStr">
         <is>
           <t>GENECIR</t>
         </is>
       </c>
-      <c r="B78" s="45" t="inlineStr">
+      <c r="B78" s="47" t="inlineStr">
         <is>
           <t>LÍQUIDO A RECEBER</t>
         </is>
       </c>
-      <c r="C78" s="45" t="inlineStr">
+      <c r="C78" s="47" t="inlineStr">
         <is>
           <t>Líquido</t>
         </is>
       </c>
-      <c r="D78" s="46">
-        <f>'HOLERITE AGO.26'!D33</f>
-        <v/>
-      </c>
-      <c r="E78" s="47" t="n"/>
+      <c r="D78" s="48">
+        <f>'HOLERITE AGO.26'!D36</f>
+        <v/>
+      </c>
+      <c r="E78" s="49" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="30" t="inlineStr">
@@ -5513,7 +5703,7 @@
         <f>'HOLERITE AGO.26'!E6</f>
         <v/>
       </c>
-      <c r="E80" s="41" t="n"/>
+      <c r="E80" s="43" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="30" t="inlineStr">
@@ -5535,7 +5725,7 @@
         <f>'HOLERITE AGO.26'!E7</f>
         <v/>
       </c>
-      <c r="E81" s="41" t="n"/>
+      <c r="E81" s="43" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="30" t="inlineStr">
@@ -5557,7 +5747,7 @@
         <f>'HOLERITE AGO.26'!E8</f>
         <v/>
       </c>
-      <c r="E82" s="41" t="n"/>
+      <c r="E82" s="43" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="30" t="inlineStr">
@@ -5579,7 +5769,7 @@
         <f>'HOLERITE AGO.26'!E11</f>
         <v/>
       </c>
-      <c r="E83" s="41" t="n"/>
+      <c r="E83" s="43" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="30" t="inlineStr">
@@ -5601,7 +5791,7 @@
         <f>'HOLERITE AGO.26'!E12</f>
         <v/>
       </c>
-      <c r="E84" s="41" t="n"/>
+      <c r="E84" s="43" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="30" t="inlineStr">
@@ -5620,10 +5810,10 @@
         </is>
       </c>
       <c r="D85" s="34">
-        <f>'HOLERITE AGO.26'!E13</f>
-        <v/>
-      </c>
-      <c r="E85" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!E16</f>
+        <v/>
+      </c>
+      <c r="E85" s="43" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="30" t="inlineStr">
@@ -5642,10 +5832,10 @@
         </is>
       </c>
       <c r="D86" s="34">
-        <f>'HOLERITE AGO.26'!E14</f>
-        <v/>
-      </c>
-      <c r="E86" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!E17</f>
+        <v/>
+      </c>
+      <c r="E86" s="43" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="30" t="inlineStr">
@@ -5664,10 +5854,10 @@
         </is>
       </c>
       <c r="D87" s="34">
-        <f>'HOLERITE AGO.26'!E15</f>
-        <v/>
-      </c>
-      <c r="E87" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!E18</f>
+        <v/>
+      </c>
+      <c r="E87" s="43" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="30" t="inlineStr">
@@ -5686,10 +5876,10 @@
         </is>
       </c>
       <c r="D88" s="34">
-        <f>'HOLERITE AGO.26'!E16</f>
-        <v/>
-      </c>
-      <c r="E88" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!E19</f>
+        <v/>
+      </c>
+      <c r="E88" s="43" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="30" t="inlineStr">
@@ -5708,10 +5898,10 @@
         </is>
       </c>
       <c r="D89" s="34">
-        <f>'HOLERITE AGO.26'!E17</f>
-        <v/>
-      </c>
-      <c r="E89" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!E20</f>
+        <v/>
+      </c>
+      <c r="E89" s="43" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="30" t="inlineStr">
@@ -5730,10 +5920,10 @@
         </is>
       </c>
       <c r="D90" s="34">
-        <f>'HOLERITE AGO.26'!E18</f>
-        <v/>
-      </c>
-      <c r="E90" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!E21</f>
+        <v/>
+      </c>
+      <c r="E90" s="43" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="30" t="inlineStr">
@@ -5752,10 +5942,10 @@
         </is>
       </c>
       <c r="D91" s="34">
-        <f>'HOLERITE AGO.26'!E19</f>
-        <v/>
-      </c>
-      <c r="E91" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!E22</f>
+        <v/>
+      </c>
+      <c r="E91" s="43" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="30" t="inlineStr">
@@ -5774,10 +5964,10 @@
         </is>
       </c>
       <c r="D92" s="34">
-        <f>'HOLERITE AGO.26'!E20</f>
-        <v/>
-      </c>
-      <c r="E92" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!E23</f>
+        <v/>
+      </c>
+      <c r="E92" s="43" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="30" t="inlineStr">
@@ -5796,29 +5986,29 @@
         </is>
       </c>
       <c r="D93" s="34">
-        <f>'HOLERITE AGO.26'!E21</f>
-        <v/>
-      </c>
-      <c r="E93" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!E24</f>
+        <v/>
+      </c>
+      <c r="E93" s="43" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="42" t="inlineStr">
+      <c r="A94" s="44" t="inlineStr">
         <is>
           <t>RENALDO</t>
         </is>
       </c>
-      <c r="B94" s="42" t="inlineStr">
+      <c r="B94" s="44" t="inlineStr">
         <is>
           <t>TOTAL DE PROVENTOS</t>
         </is>
       </c>
-      <c r="C94" s="42" t="inlineStr">
+      <c r="C94" s="44" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="D94" s="43">
-        <f>'HOLERITE AGO.26'!E22</f>
+      <c r="D94" s="45">
+        <f>'HOLERITE AGO.26'!E25</f>
         <v/>
       </c>
       <c r="E94" s="18" t="n"/>
@@ -5840,10 +6030,10 @@
         </is>
       </c>
       <c r="D95" s="34">
-        <f>'HOLERITE AGO.26'!E24</f>
-        <v/>
-      </c>
-      <c r="E95" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!E27</f>
+        <v/>
+      </c>
+      <c r="E95" s="43" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="30" t="inlineStr">
@@ -5862,10 +6052,10 @@
         </is>
       </c>
       <c r="D96" s="34">
-        <f>'HOLERITE AGO.26'!E25</f>
-        <v/>
-      </c>
-      <c r="E96" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!E28</f>
+        <v/>
+      </c>
+      <c r="E96" s="43" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="30" t="inlineStr">
@@ -5884,10 +6074,10 @@
         </is>
       </c>
       <c r="D97" s="34">
-        <f>'HOLERITE AGO.26'!E26</f>
-        <v/>
-      </c>
-      <c r="E97" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!E29</f>
+        <v/>
+      </c>
+      <c r="E97" s="43" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="30" t="inlineStr">
@@ -5906,10 +6096,10 @@
         </is>
       </c>
       <c r="D98" s="34">
-        <f>'HOLERITE AGO.26'!E27</f>
-        <v/>
-      </c>
-      <c r="E98" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!E30</f>
+        <v/>
+      </c>
+      <c r="E98" s="43" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="30" t="inlineStr">
@@ -5928,10 +6118,10 @@
         </is>
       </c>
       <c r="D99" s="34">
-        <f>'HOLERITE AGO.26'!E28</f>
-        <v/>
-      </c>
-      <c r="E99" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!E31</f>
+        <v/>
+      </c>
+      <c r="E99" s="43" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="30" t="inlineStr">
@@ -5950,10 +6140,10 @@
         </is>
       </c>
       <c r="D100" s="34">
-        <f>'HOLERITE AGO.26'!E29</f>
-        <v/>
-      </c>
-      <c r="E100" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!E32</f>
+        <v/>
+      </c>
+      <c r="E100" s="43" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="30" t="inlineStr">
@@ -5972,54 +6162,54 @@
         </is>
       </c>
       <c r="D101" s="34">
-        <f>'HOLERITE AGO.26'!E30</f>
-        <v/>
-      </c>
-      <c r="E101" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!E33</f>
+        <v/>
+      </c>
+      <c r="E101" s="43" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="42" t="inlineStr">
+      <c r="A102" s="44" t="inlineStr">
         <is>
           <t>RENALDO</t>
         </is>
       </c>
-      <c r="B102" s="42" t="inlineStr">
+      <c r="B102" s="44" t="inlineStr">
         <is>
           <t>TOTAL DE DESCONTOS</t>
         </is>
       </c>
-      <c r="C102" s="42" t="inlineStr">
+      <c r="C102" s="44" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="D102" s="43">
-        <f>'HOLERITE AGO.26'!E31</f>
+      <c r="D102" s="45">
+        <f>'HOLERITE AGO.26'!E34</f>
         <v/>
       </c>
       <c r="E102" s="18" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="44" t="inlineStr">
+      <c r="A103" s="46" t="inlineStr">
         <is>
           <t>RENALDO</t>
         </is>
       </c>
-      <c r="B103" s="45" t="inlineStr">
+      <c r="B103" s="47" t="inlineStr">
         <is>
           <t>LÍQUIDO A RECEBER</t>
         </is>
       </c>
-      <c r="C103" s="45" t="inlineStr">
+      <c r="C103" s="47" t="inlineStr">
         <is>
           <t>Líquido</t>
         </is>
       </c>
-      <c r="D103" s="46">
-        <f>'HOLERITE AGO.26'!E33</f>
-        <v/>
-      </c>
-      <c r="E103" s="47" t="n"/>
+      <c r="D103" s="48">
+        <f>'HOLERITE AGO.26'!E36</f>
+        <v/>
+      </c>
+      <c r="E103" s="49" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="30" t="inlineStr">
@@ -6041,7 +6231,7 @@
         <f>'HOLERITE AGO.26'!F6</f>
         <v/>
       </c>
-      <c r="E105" s="41" t="n"/>
+      <c r="E105" s="43" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="30" t="inlineStr">
@@ -6063,7 +6253,7 @@
         <f>'HOLERITE AGO.26'!F7</f>
         <v/>
       </c>
-      <c r="E106" s="41" t="n"/>
+      <c r="E106" s="43" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="30" t="inlineStr">
@@ -6085,7 +6275,7 @@
         <f>'HOLERITE AGO.26'!F8</f>
         <v/>
       </c>
-      <c r="E107" s="41" t="n"/>
+      <c r="E107" s="43" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="30" t="inlineStr">
@@ -6107,7 +6297,7 @@
         <f>'HOLERITE AGO.26'!F11</f>
         <v/>
       </c>
-      <c r="E108" s="41" t="n"/>
+      <c r="E108" s="43" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="30" t="inlineStr">
@@ -6129,7 +6319,7 @@
         <f>'HOLERITE AGO.26'!F12</f>
         <v/>
       </c>
-      <c r="E109" s="41" t="n"/>
+      <c r="E109" s="43" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="30" t="inlineStr">
@@ -6148,10 +6338,10 @@
         </is>
       </c>
       <c r="D110" s="34">
-        <f>'HOLERITE AGO.26'!F13</f>
-        <v/>
-      </c>
-      <c r="E110" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!F16</f>
+        <v/>
+      </c>
+      <c r="E110" s="43" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="30" t="inlineStr">
@@ -6170,10 +6360,10 @@
         </is>
       </c>
       <c r="D111" s="34">
-        <f>'HOLERITE AGO.26'!F14</f>
-        <v/>
-      </c>
-      <c r="E111" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!F17</f>
+        <v/>
+      </c>
+      <c r="E111" s="43" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="30" t="inlineStr">
@@ -6192,10 +6382,10 @@
         </is>
       </c>
       <c r="D112" s="34">
-        <f>'HOLERITE AGO.26'!F15</f>
-        <v/>
-      </c>
-      <c r="E112" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!F18</f>
+        <v/>
+      </c>
+      <c r="E112" s="43" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="30" t="inlineStr">
@@ -6214,10 +6404,10 @@
         </is>
       </c>
       <c r="D113" s="34">
-        <f>'HOLERITE AGO.26'!F16</f>
-        <v/>
-      </c>
-      <c r="E113" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!F19</f>
+        <v/>
+      </c>
+      <c r="E113" s="43" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="30" t="inlineStr">
@@ -6236,10 +6426,10 @@
         </is>
       </c>
       <c r="D114" s="34">
-        <f>'HOLERITE AGO.26'!F17</f>
-        <v/>
-      </c>
-      <c r="E114" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!F20</f>
+        <v/>
+      </c>
+      <c r="E114" s="43" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="30" t="inlineStr">
@@ -6258,10 +6448,10 @@
         </is>
       </c>
       <c r="D115" s="34">
-        <f>'HOLERITE AGO.26'!F18</f>
-        <v/>
-      </c>
-      <c r="E115" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!F21</f>
+        <v/>
+      </c>
+      <c r="E115" s="43" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="30" t="inlineStr">
@@ -6280,10 +6470,10 @@
         </is>
       </c>
       <c r="D116" s="34">
-        <f>'HOLERITE AGO.26'!F19</f>
-        <v/>
-      </c>
-      <c r="E116" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!F22</f>
+        <v/>
+      </c>
+      <c r="E116" s="43" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="30" t="inlineStr">
@@ -6302,10 +6492,10 @@
         </is>
       </c>
       <c r="D117" s="34">
-        <f>'HOLERITE AGO.26'!F20</f>
-        <v/>
-      </c>
-      <c r="E117" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!F23</f>
+        <v/>
+      </c>
+      <c r="E117" s="43" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="30" t="inlineStr">
@@ -6324,29 +6514,29 @@
         </is>
       </c>
       <c r="D118" s="34">
-        <f>'HOLERITE AGO.26'!F21</f>
-        <v/>
-      </c>
-      <c r="E118" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!F24</f>
+        <v/>
+      </c>
+      <c r="E118" s="43" t="n"/>
     </row>
     <row r="119">
-      <c r="A119" s="42" t="inlineStr">
+      <c r="A119" s="44" t="inlineStr">
         <is>
           <t>THAYANE</t>
         </is>
       </c>
-      <c r="B119" s="42" t="inlineStr">
+      <c r="B119" s="44" t="inlineStr">
         <is>
           <t>TOTAL DE PROVENTOS</t>
         </is>
       </c>
-      <c r="C119" s="42" t="inlineStr">
+      <c r="C119" s="44" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="D119" s="43">
-        <f>'HOLERITE AGO.26'!F22</f>
+      <c r="D119" s="45">
+        <f>'HOLERITE AGO.26'!F25</f>
         <v/>
       </c>
       <c r="E119" s="18" t="n"/>
@@ -6368,10 +6558,10 @@
         </is>
       </c>
       <c r="D120" s="34">
-        <f>'HOLERITE AGO.26'!F24</f>
-        <v/>
-      </c>
-      <c r="E120" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!F27</f>
+        <v/>
+      </c>
+      <c r="E120" s="43" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="30" t="inlineStr">
@@ -6390,10 +6580,10 @@
         </is>
       </c>
       <c r="D121" s="34">
-        <f>'HOLERITE AGO.26'!F25</f>
-        <v/>
-      </c>
-      <c r="E121" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!F28</f>
+        <v/>
+      </c>
+      <c r="E121" s="43" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="30" t="inlineStr">
@@ -6412,10 +6602,10 @@
         </is>
       </c>
       <c r="D122" s="34">
-        <f>'HOLERITE AGO.26'!F26</f>
-        <v/>
-      </c>
-      <c r="E122" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!F29</f>
+        <v/>
+      </c>
+      <c r="E122" s="43" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="30" t="inlineStr">
@@ -6434,10 +6624,10 @@
         </is>
       </c>
       <c r="D123" s="34">
-        <f>'HOLERITE AGO.26'!F27</f>
-        <v/>
-      </c>
-      <c r="E123" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!F30</f>
+        <v/>
+      </c>
+      <c r="E123" s="43" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="30" t="inlineStr">
@@ -6456,10 +6646,10 @@
         </is>
       </c>
       <c r="D124" s="34">
-        <f>'HOLERITE AGO.26'!F28</f>
-        <v/>
-      </c>
-      <c r="E124" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!F31</f>
+        <v/>
+      </c>
+      <c r="E124" s="43" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="30" t="inlineStr">
@@ -6478,10 +6668,10 @@
         </is>
       </c>
       <c r="D125" s="34">
-        <f>'HOLERITE AGO.26'!F29</f>
-        <v/>
-      </c>
-      <c r="E125" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!F32</f>
+        <v/>
+      </c>
+      <c r="E125" s="43" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="30" t="inlineStr">
@@ -6500,54 +6690,54 @@
         </is>
       </c>
       <c r="D126" s="34">
-        <f>'HOLERITE AGO.26'!F30</f>
-        <v/>
-      </c>
-      <c r="E126" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!F33</f>
+        <v/>
+      </c>
+      <c r="E126" s="43" t="n"/>
     </row>
     <row r="127">
-      <c r="A127" s="42" t="inlineStr">
+      <c r="A127" s="44" t="inlineStr">
         <is>
           <t>THAYANE</t>
         </is>
       </c>
-      <c r="B127" s="42" t="inlineStr">
+      <c r="B127" s="44" t="inlineStr">
         <is>
           <t>TOTAL DE DESCONTOS</t>
         </is>
       </c>
-      <c r="C127" s="42" t="inlineStr">
+      <c r="C127" s="44" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="D127" s="43">
-        <f>'HOLERITE AGO.26'!F31</f>
+      <c r="D127" s="45">
+        <f>'HOLERITE AGO.26'!F34</f>
         <v/>
       </c>
       <c r="E127" s="18" t="n"/>
     </row>
     <row r="128">
-      <c r="A128" s="44" t="inlineStr">
+      <c r="A128" s="46" t="inlineStr">
         <is>
           <t>THAYANE</t>
         </is>
       </c>
-      <c r="B128" s="45" t="inlineStr">
+      <c r="B128" s="47" t="inlineStr">
         <is>
           <t>LÍQUIDO A RECEBER</t>
         </is>
       </c>
-      <c r="C128" s="45" t="inlineStr">
+      <c r="C128" s="47" t="inlineStr">
         <is>
           <t>Líquido</t>
         </is>
       </c>
-      <c r="D128" s="46">
-        <f>'HOLERITE AGO.26'!F33</f>
-        <v/>
-      </c>
-      <c r="E128" s="47" t="n"/>
+      <c r="D128" s="48">
+        <f>'HOLERITE AGO.26'!F36</f>
+        <v/>
+      </c>
+      <c r="E128" s="49" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="30" t="inlineStr">
@@ -6569,7 +6759,7 @@
         <f>'HOLERITE AGO.26'!G6</f>
         <v/>
       </c>
-      <c r="E130" s="41" t="n"/>
+      <c r="E130" s="43" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="30" t="inlineStr">
@@ -6591,7 +6781,7 @@
         <f>'HOLERITE AGO.26'!G7</f>
         <v/>
       </c>
-      <c r="E131" s="41" t="n"/>
+      <c r="E131" s="43" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="30" t="inlineStr">
@@ -6613,7 +6803,7 @@
         <f>'HOLERITE AGO.26'!G8</f>
         <v/>
       </c>
-      <c r="E132" s="41" t="n"/>
+      <c r="E132" s="43" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="30" t="inlineStr">
@@ -6635,7 +6825,7 @@
         <f>'HOLERITE AGO.26'!G11</f>
         <v/>
       </c>
-      <c r="E133" s="41" t="n"/>
+      <c r="E133" s="43" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="30" t="inlineStr">
@@ -6657,7 +6847,7 @@
         <f>'HOLERITE AGO.26'!G12</f>
         <v/>
       </c>
-      <c r="E134" s="41" t="n"/>
+      <c r="E134" s="43" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="30" t="inlineStr">
@@ -6676,10 +6866,10 @@
         </is>
       </c>
       <c r="D135" s="34">
-        <f>'HOLERITE AGO.26'!G13</f>
-        <v/>
-      </c>
-      <c r="E135" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!G16</f>
+        <v/>
+      </c>
+      <c r="E135" s="43" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="30" t="inlineStr">
@@ -6698,10 +6888,10 @@
         </is>
       </c>
       <c r="D136" s="34">
-        <f>'HOLERITE AGO.26'!G14</f>
-        <v/>
-      </c>
-      <c r="E136" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!G17</f>
+        <v/>
+      </c>
+      <c r="E136" s="43" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="30" t="inlineStr">
@@ -6720,10 +6910,10 @@
         </is>
       </c>
       <c r="D137" s="34">
-        <f>'HOLERITE AGO.26'!G15</f>
-        <v/>
-      </c>
-      <c r="E137" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!G18</f>
+        <v/>
+      </c>
+      <c r="E137" s="43" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="30" t="inlineStr">
@@ -6742,10 +6932,10 @@
         </is>
       </c>
       <c r="D138" s="34">
-        <f>'HOLERITE AGO.26'!G16</f>
-        <v/>
-      </c>
-      <c r="E138" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!G19</f>
+        <v/>
+      </c>
+      <c r="E138" s="43" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="30" t="inlineStr">
@@ -6764,10 +6954,10 @@
         </is>
       </c>
       <c r="D139" s="34">
-        <f>'HOLERITE AGO.26'!G17</f>
-        <v/>
-      </c>
-      <c r="E139" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!G20</f>
+        <v/>
+      </c>
+      <c r="E139" s="43" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="30" t="inlineStr">
@@ -6786,10 +6976,10 @@
         </is>
       </c>
       <c r="D140" s="34">
-        <f>'HOLERITE AGO.26'!G18</f>
-        <v/>
-      </c>
-      <c r="E140" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!G21</f>
+        <v/>
+      </c>
+      <c r="E140" s="43" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="30" t="inlineStr">
@@ -6808,10 +6998,10 @@
         </is>
       </c>
       <c r="D141" s="34">
-        <f>'HOLERITE AGO.26'!G19</f>
-        <v/>
-      </c>
-      <c r="E141" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!G22</f>
+        <v/>
+      </c>
+      <c r="E141" s="43" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="30" t="inlineStr">
@@ -6830,10 +7020,10 @@
         </is>
       </c>
       <c r="D142" s="34">
-        <f>'HOLERITE AGO.26'!G20</f>
-        <v/>
-      </c>
-      <c r="E142" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!G23</f>
+        <v/>
+      </c>
+      <c r="E142" s="43" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="30" t="inlineStr">
@@ -6852,29 +7042,29 @@
         </is>
       </c>
       <c r="D143" s="34">
-        <f>'HOLERITE AGO.26'!G21</f>
-        <v/>
-      </c>
-      <c r="E143" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!G24</f>
+        <v/>
+      </c>
+      <c r="E143" s="43" t="n"/>
     </row>
     <row r="144">
-      <c r="A144" s="42" t="inlineStr">
+      <c r="A144" s="44" t="inlineStr">
         <is>
           <t>PEDRO</t>
         </is>
       </c>
-      <c r="B144" s="42" t="inlineStr">
+      <c r="B144" s="44" t="inlineStr">
         <is>
           <t>TOTAL DE PROVENTOS</t>
         </is>
       </c>
-      <c r="C144" s="42" t="inlineStr">
+      <c r="C144" s="44" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="D144" s="43">
-        <f>'HOLERITE AGO.26'!G22</f>
+      <c r="D144" s="45">
+        <f>'HOLERITE AGO.26'!G25</f>
         <v/>
       </c>
       <c r="E144" s="18" t="n"/>
@@ -6896,10 +7086,10 @@
         </is>
       </c>
       <c r="D145" s="34">
-        <f>'HOLERITE AGO.26'!G24</f>
-        <v/>
-      </c>
-      <c r="E145" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!G27</f>
+        <v/>
+      </c>
+      <c r="E145" s="43" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="30" t="inlineStr">
@@ -6918,10 +7108,10 @@
         </is>
       </c>
       <c r="D146" s="34">
-        <f>'HOLERITE AGO.26'!G25</f>
-        <v/>
-      </c>
-      <c r="E146" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!G28</f>
+        <v/>
+      </c>
+      <c r="E146" s="43" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="30" t="inlineStr">
@@ -6940,10 +7130,10 @@
         </is>
       </c>
       <c r="D147" s="34">
-        <f>'HOLERITE AGO.26'!G26</f>
-        <v/>
-      </c>
-      <c r="E147" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!G29</f>
+        <v/>
+      </c>
+      <c r="E147" s="43" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="30" t="inlineStr">
@@ -6962,10 +7152,10 @@
         </is>
       </c>
       <c r="D148" s="34">
-        <f>'HOLERITE AGO.26'!G27</f>
-        <v/>
-      </c>
-      <c r="E148" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!G30</f>
+        <v/>
+      </c>
+      <c r="E148" s="43" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="30" t="inlineStr">
@@ -6984,10 +7174,10 @@
         </is>
       </c>
       <c r="D149" s="34">
-        <f>'HOLERITE AGO.26'!G28</f>
-        <v/>
-      </c>
-      <c r="E149" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!G31</f>
+        <v/>
+      </c>
+      <c r="E149" s="43" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="30" t="inlineStr">
@@ -7006,10 +7196,10 @@
         </is>
       </c>
       <c r="D150" s="34">
-        <f>'HOLERITE AGO.26'!G29</f>
-        <v/>
-      </c>
-      <c r="E150" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!G32</f>
+        <v/>
+      </c>
+      <c r="E150" s="43" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="30" t="inlineStr">
@@ -7028,54 +7218,54 @@
         </is>
       </c>
       <c r="D151" s="34">
-        <f>'HOLERITE AGO.26'!G30</f>
-        <v/>
-      </c>
-      <c r="E151" s="41" t="n"/>
+        <f>'HOLERITE AGO.26'!G33</f>
+        <v/>
+      </c>
+      <c r="E151" s="43" t="n"/>
     </row>
     <row r="152">
-      <c r="A152" s="42" t="inlineStr">
+      <c r="A152" s="44" t="inlineStr">
         <is>
           <t>PEDRO</t>
         </is>
       </c>
-      <c r="B152" s="42" t="inlineStr">
+      <c r="B152" s="44" t="inlineStr">
         <is>
           <t>TOTAL DE DESCONTOS</t>
         </is>
       </c>
-      <c r="C152" s="42" t="inlineStr">
+      <c r="C152" s="44" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="D152" s="43">
-        <f>'HOLERITE AGO.26'!G31</f>
+      <c r="D152" s="45">
+        <f>'HOLERITE AGO.26'!G34</f>
         <v/>
       </c>
       <c r="E152" s="18" t="n"/>
     </row>
     <row r="153">
-      <c r="A153" s="44" t="inlineStr">
+      <c r="A153" s="46" t="inlineStr">
         <is>
           <t>PEDRO</t>
         </is>
       </c>
-      <c r="B153" s="45" t="inlineStr">
+      <c r="B153" s="47" t="inlineStr">
         <is>
           <t>LÍQUIDO A RECEBER</t>
         </is>
       </c>
-      <c r="C153" s="45" t="inlineStr">
+      <c r="C153" s="47" t="inlineStr">
         <is>
           <t>Líquido</t>
         </is>
       </c>
-      <c r="D153" s="46">
-        <f>'HOLERITE AGO.26'!G33</f>
-        <v/>
-      </c>
-      <c r="E153" s="47" t="n"/>
+      <c r="D153" s="48">
+        <f>'HOLERITE AGO.26'!G36</f>
+        <v/>
+      </c>
+      <c r="E153" s="49" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:E153"/>
@@ -7117,12 +7307,12 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="48" t="inlineStr">
+      <c r="B4" s="50" t="inlineStr">
         <is>
           <t>Escolha o colaborador:</t>
         </is>
       </c>
-      <c r="C4" s="49" t="inlineStr">
+      <c r="C4" s="51" t="inlineStr">
         <is>
           <t>ARIANE</t>
         </is>
@@ -7204,7 +7394,7 @@
         </is>
       </c>
       <c r="C12" s="34">
-        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$13:$G$13,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$16:$G$16,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
     </row>
@@ -7215,7 +7405,7 @@
         </is>
       </c>
       <c r="C13" s="34">
-        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$14:$G$14,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$17:$G$17,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
     </row>
@@ -7226,7 +7416,7 @@
         </is>
       </c>
       <c r="C14" s="34">
-        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$15:$G$15,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$18:$G$18,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
     </row>
@@ -7237,7 +7427,7 @@
         </is>
       </c>
       <c r="C15" s="34">
-        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$16:$G$16,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$19:$G$19,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
     </row>
@@ -7248,7 +7438,7 @@
         </is>
       </c>
       <c r="C16" s="34">
-        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$17:$G$17,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$20:$G$20,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
     </row>
@@ -7259,7 +7449,7 @@
         </is>
       </c>
       <c r="C17" s="34">
-        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$18:$G$18,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$21:$G$21,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
     </row>
@@ -7270,7 +7460,7 @@
         </is>
       </c>
       <c r="C18" s="34">
-        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$19:$G$19,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$22:$G$22,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
     </row>
@@ -7281,7 +7471,7 @@
         </is>
       </c>
       <c r="C19" s="34">
-        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$20:$G$20,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$23:$G$23,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
     </row>
@@ -7292,7 +7482,7 @@
         </is>
       </c>
       <c r="C20" s="34">
-        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$21:$G$21,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$24:$G$24,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
     </row>
@@ -7302,8 +7492,8 @@
           <t>TOTAL DE PROVENTOS</t>
         </is>
       </c>
-      <c r="C21" s="43">
-        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$22:$G$22,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
+      <c r="C21" s="45">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$25:$G$25,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
     </row>
@@ -7323,7 +7513,7 @@
         </is>
       </c>
       <c r="C23" s="34">
-        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$24:$G$24,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$27:$G$27,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
     </row>
@@ -7334,7 +7524,7 @@
         </is>
       </c>
       <c r="C24" s="34">
-        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$25:$G$25,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$28:$G$28,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
     </row>
@@ -7345,7 +7535,7 @@
         </is>
       </c>
       <c r="C25" s="34">
-        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$26:$G$26,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$29:$G$29,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
     </row>
@@ -7356,7 +7546,7 @@
         </is>
       </c>
       <c r="C26" s="34">
-        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$27:$G$27,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$30:$G$30,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
     </row>
@@ -7367,7 +7557,7 @@
         </is>
       </c>
       <c r="C27" s="34">
-        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$28:$G$28,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$31:$G$31,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
     </row>
@@ -7378,7 +7568,7 @@
         </is>
       </c>
       <c r="C28" s="34">
-        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$29:$G$29,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$32:$G$32,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
     </row>
@@ -7389,7 +7579,7 @@
         </is>
       </c>
       <c r="C29" s="34">
-        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$30:$G$30,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$33:$G$33,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
     </row>
@@ -7399,8 +7589,8 @@
           <t>TOTAL DE DESCONTOS</t>
         </is>
       </c>
-      <c r="C30" s="43">
-        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$31:$G$31,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
+      <c r="C30" s="45">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$34:$G$34,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
     </row>
@@ -7414,18 +7604,18 @@
       <c r="D31" s="29" t="n"/>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="B32" s="50" t="inlineStr">
+      <c r="B32" s="52" t="inlineStr">
         <is>
           <t>LÍQUIDO A RECEBER EM 05/09/2026</t>
         </is>
       </c>
-      <c r="C32" s="51">
-        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$33:$G$33,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
+      <c r="C32" s="53">
+        <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$36:$G$36,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="52" t="inlineStr">
+      <c r="B34" s="54" t="inlineStr">
         <is>
           <t>Vendas do colaborador no mês (InovaFarma):</t>
         </is>
@@ -7604,10 +7794,10 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="53" t="n"/>
-      <c r="B5" s="53" t="n"/>
-      <c r="C5" s="53" t="n"/>
-      <c r="D5" s="53" t="n"/>
+      <c r="A5" s="55" t="n"/>
+      <c r="B5" s="55" t="n"/>
+      <c r="C5" s="55" t="n"/>
+      <c r="D5" s="55" t="n"/>
       <c r="E5" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$6:$G$6,1,MATCH(A5,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
@@ -7617,14 +7807,14 @@
         <f>ROUND(C5*F5,2)</f>
         <v/>
       </c>
-      <c r="H5" s="53" t="n"/>
-      <c r="I5" s="53" t="n"/>
+      <c r="H5" s="55" t="n"/>
+      <c r="I5" s="55" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="53" t="n"/>
-      <c r="B6" s="53" t="n"/>
-      <c r="C6" s="53" t="n"/>
-      <c r="D6" s="53" t="n"/>
+      <c r="A6" s="55" t="n"/>
+      <c r="B6" s="55" t="n"/>
+      <c r="C6" s="55" t="n"/>
+      <c r="D6" s="55" t="n"/>
       <c r="E6" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$6:$G$6,1,MATCH(A6,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
@@ -7634,14 +7824,14 @@
         <f>ROUND(C6*F6,2)</f>
         <v/>
       </c>
-      <c r="H6" s="53" t="n"/>
-      <c r="I6" s="53" t="n"/>
+      <c r="H6" s="55" t="n"/>
+      <c r="I6" s="55" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="53" t="n"/>
-      <c r="B7" s="53" t="n"/>
-      <c r="C7" s="53" t="n"/>
-      <c r="D7" s="53" t="n"/>
+      <c r="A7" s="55" t="n"/>
+      <c r="B7" s="55" t="n"/>
+      <c r="C7" s="55" t="n"/>
+      <c r="D7" s="55" t="n"/>
       <c r="E7" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$6:$G$6,1,MATCH(A7,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
@@ -7651,14 +7841,14 @@
         <f>ROUND(C7*F7,2)</f>
         <v/>
       </c>
-      <c r="H7" s="53" t="n"/>
-      <c r="I7" s="53" t="n"/>
+      <c r="H7" s="55" t="n"/>
+      <c r="I7" s="55" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="53" t="n"/>
-      <c r="B8" s="53" t="n"/>
-      <c r="C8" s="53" t="n"/>
-      <c r="D8" s="53" t="n"/>
+      <c r="A8" s="55" t="n"/>
+      <c r="B8" s="55" t="n"/>
+      <c r="C8" s="55" t="n"/>
+      <c r="D8" s="55" t="n"/>
       <c r="E8" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$6:$G$6,1,MATCH(A8,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
@@ -7668,14 +7858,14 @@
         <f>ROUND(C8*F8,2)</f>
         <v/>
       </c>
-      <c r="H8" s="53" t="n"/>
-      <c r="I8" s="53" t="n"/>
+      <c r="H8" s="55" t="n"/>
+      <c r="I8" s="55" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="53" t="n"/>
-      <c r="B9" s="53" t="n"/>
-      <c r="C9" s="53" t="n"/>
-      <c r="D9" s="53" t="n"/>
+      <c r="A9" s="55" t="n"/>
+      <c r="B9" s="55" t="n"/>
+      <c r="C9" s="55" t="n"/>
+      <c r="D9" s="55" t="n"/>
       <c r="E9" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$6:$G$6,1,MATCH(A9,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
@@ -7685,14 +7875,14 @@
         <f>ROUND(C9*F9,2)</f>
         <v/>
       </c>
-      <c r="H9" s="53" t="n"/>
-      <c r="I9" s="53" t="n"/>
+      <c r="H9" s="55" t="n"/>
+      <c r="I9" s="55" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="53" t="n"/>
-      <c r="B10" s="53" t="n"/>
-      <c r="C10" s="53" t="n"/>
-      <c r="D10" s="53" t="n"/>
+      <c r="A10" s="55" t="n"/>
+      <c r="B10" s="55" t="n"/>
+      <c r="C10" s="55" t="n"/>
+      <c r="D10" s="55" t="n"/>
       <c r="E10" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$6:$G$6,1,MATCH(A10,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
@@ -7702,14 +7892,14 @@
         <f>ROUND(C10*F10,2)</f>
         <v/>
       </c>
-      <c r="H10" s="53" t="n"/>
-      <c r="I10" s="53" t="n"/>
+      <c r="H10" s="55" t="n"/>
+      <c r="I10" s="55" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="53" t="n"/>
-      <c r="B11" s="53" t="n"/>
-      <c r="C11" s="53" t="n"/>
-      <c r="D11" s="53" t="n"/>
+      <c r="A11" s="55" t="n"/>
+      <c r="B11" s="55" t="n"/>
+      <c r="C11" s="55" t="n"/>
+      <c r="D11" s="55" t="n"/>
       <c r="E11" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$6:$G$6,1,MATCH(A11,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
@@ -7719,14 +7909,14 @@
         <f>ROUND(C11*F11,2)</f>
         <v/>
       </c>
-      <c r="H11" s="53" t="n"/>
-      <c r="I11" s="53" t="n"/>
+      <c r="H11" s="55" t="n"/>
+      <c r="I11" s="55" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="53" t="n"/>
-      <c r="B12" s="53" t="n"/>
-      <c r="C12" s="53" t="n"/>
-      <c r="D12" s="53" t="n"/>
+      <c r="A12" s="55" t="n"/>
+      <c r="B12" s="55" t="n"/>
+      <c r="C12" s="55" t="n"/>
+      <c r="D12" s="55" t="n"/>
       <c r="E12" s="34">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$6:$G$6,1,MATCH(A12,'HOLERITE AGO.26'!$B$4:$G$4,0)),0)</f>
         <v/>
@@ -7736,8 +7926,8 @@
         <f>ROUND(C12*F12,2)</f>
         <v/>
       </c>
-      <c r="H12" s="53" t="n"/>
-      <c r="I12" s="53" t="n"/>
+      <c r="H12" s="55" t="n"/>
+      <c r="I12" s="55" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="18" t="n"/>
@@ -7889,7 +8079,7 @@
         <v>150</v>
       </c>
       <c r="D5" s="8" t="n"/>
-      <c r="E5" s="54">
+      <c r="E5" s="56">
         <f>C5*D5</f>
         <v/>
       </c>
@@ -7899,7 +8089,7 @@
       <c r="G5" s="35" t="n">
         <v>40</v>
       </c>
-      <c r="H5" s="38">
+      <c r="H5" s="40">
         <f>E5+F5+G5</f>
         <v/>
       </c>
@@ -7919,7 +8109,7 @@
         <v>100</v>
       </c>
       <c r="D6" s="8" t="n"/>
-      <c r="E6" s="54">
+      <c r="E6" s="56">
         <f>C6*D6</f>
         <v/>
       </c>
@@ -7929,7 +8119,7 @@
       <c r="G6" s="35" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="38">
+      <c r="H6" s="40">
         <f>E6+F6+G6</f>
         <v/>
       </c>

</xml_diff>